<commit_message>
chore: update Sheets via scheduled runner
</commit_message>
<xml_diff>
--- a/Sheets/Adamantoise_Profits.xlsx
+++ b/Sheets/Adamantoise_Profits.xlsx
@@ -912,25 +912,25 @@
         <v>4564</v>
       </c>
       <c r="H6" t="n">
-        <v>18272842</v>
+        <v>20000224</v>
       </c>
       <c r="I6" t="n">
-        <v>20000126</v>
+        <v>22222360</v>
       </c>
       <c r="J6" t="n">
-        <v>1000000</v>
+        <v>1000</v>
       </c>
       <c r="K6" t="n">
-        <v>60000378</v>
+        <v>66667080</v>
       </c>
       <c r="L6" t="n">
-        <v>3000000</v>
+        <v>3000</v>
       </c>
       <c r="M6" t="n">
-        <v>-60000266</v>
+        <v>-66666968</v>
       </c>
       <c r="N6" t="n">
-        <v>-3000224</v>
+        <v>-3224</v>
       </c>
     </row>
     <row r="7">
@@ -1212,22 +1212,22 @@
         <v>5515</v>
       </c>
       <c r="H12" t="n">
-        <v>453.41666</v>
+        <v>447.54544</v>
       </c>
       <c r="I12" t="n">
-        <v>341.2857</v>
+        <v>311.83334</v>
       </c>
       <c r="J12" t="n">
         <v>610.4</v>
       </c>
       <c r="K12" t="n">
-        <v>341.2857</v>
+        <v>311.83334</v>
       </c>
       <c r="L12" t="n">
         <v>610.4</v>
       </c>
       <c r="M12" t="n">
-        <v>-171.2857</v>
+        <v>-141.83334</v>
       </c>
       <c r="N12" t="n">
         <v>-950.4</v>
@@ -1616,19 +1616,22 @@
         <v>1965</v>
       </c>
       <c r="H20" t="n">
-        <v>0</v>
+        <v>2000</v>
       </c>
       <c r="I20" t="n">
-        <v>0</v>
+        <v>2000</v>
       </c>
       <c r="J20" t="n">
         <v>0</v>
       </c>
       <c r="K20" t="n">
-        <v>0</v>
+        <v>2000</v>
       </c>
       <c r="L20" t="n">
         <v>0</v>
+      </c>
+      <c r="M20" t="n">
+        <v>-1770</v>
       </c>
     </row>
     <row r="21">
@@ -2336,19 +2339,22 @@
         <v>1965</v>
       </c>
       <c r="H35" t="n">
-        <v>0</v>
+        <v>2000</v>
       </c>
       <c r="I35" t="n">
-        <v>0</v>
+        <v>2000</v>
       </c>
       <c r="J35" t="n">
         <v>0</v>
       </c>
       <c r="K35" t="n">
-        <v>0</v>
+        <v>2000</v>
       </c>
       <c r="L35" t="n">
         <v>0</v>
+      </c>
+      <c r="M35" t="n">
+        <v>-1621</v>
       </c>
     </row>
     <row r="36">
@@ -2480,25 +2486,22 @@
         <v>4599</v>
       </c>
       <c r="H38" t="n">
-        <v>668</v>
+        <v>103.111115</v>
       </c>
       <c r="I38" t="n">
-        <v>126.5</v>
+        <v>103.111115</v>
       </c>
       <c r="J38" t="n">
-        <v>5000</v>
+        <v>0</v>
       </c>
       <c r="K38" t="n">
-        <v>379.5</v>
+        <v>309.333345</v>
       </c>
       <c r="L38" t="n">
-        <v>15000</v>
+        <v>0</v>
       </c>
       <c r="M38" t="n">
-        <v>-7.5</v>
-      </c>
-      <c r="N38" t="n">
-        <v>-15744</v>
+        <v>62.66665499999999</v>
       </c>
     </row>
     <row r="39">
@@ -2584,25 +2587,25 @@
         <v>5505</v>
       </c>
       <c r="H40" t="n">
-        <v>3616.1292</v>
+        <v>3675.862</v>
       </c>
       <c r="I40" t="n">
-        <v>2020</v>
+        <v>2150</v>
       </c>
       <c r="J40" t="n">
-        <v>3923.077</v>
+        <v>3920</v>
       </c>
       <c r="K40" t="n">
-        <v>2020</v>
+        <v>2150</v>
       </c>
       <c r="L40" t="n">
-        <v>3923.077</v>
+        <v>3920</v>
       </c>
       <c r="M40" t="n">
-        <v>-1845</v>
+        <v>-1975</v>
       </c>
       <c r="N40" t="n">
-        <v>-4273.077</v>
+        <v>-4270</v>
       </c>
     </row>
     <row r="41">
@@ -2740,22 +2743,22 @@
         <v>5472</v>
       </c>
       <c r="H43" t="n">
-        <v>9996.666999999999</v>
+        <v>9998.666999999999</v>
       </c>
       <c r="I43" t="n">
         <v>0</v>
       </c>
       <c r="J43" t="n">
-        <v>9996.666999999999</v>
+        <v>9998.666999999999</v>
       </c>
       <c r="K43" t="n">
         <v>0</v>
       </c>
       <c r="L43" t="n">
-        <v>9996.666999999999</v>
+        <v>9998.666999999999</v>
       </c>
       <c r="N43" t="n">
-        <v>-10134.667</v>
+        <v>-10136.667</v>
       </c>
     </row>
     <row r="44">
@@ -3132,22 +3135,19 @@
         <v>5486</v>
       </c>
       <c r="H51" t="n">
-        <v>999</v>
+        <v>0</v>
       </c>
       <c r="I51" t="n">
-        <v>999</v>
+        <v>0</v>
       </c>
       <c r="J51" t="n">
         <v>0</v>
       </c>
       <c r="K51" t="n">
-        <v>999</v>
+        <v>0</v>
       </c>
       <c r="L51" t="n">
         <v>0</v>
-      </c>
-      <c r="M51" t="n">
-        <v>-515</v>
       </c>
     </row>
     <row r="52">
@@ -3680,22 +3680,22 @@
         <v>27781</v>
       </c>
       <c r="H62" t="n">
-        <v>5295.4243</v>
+        <v>5390.25</v>
       </c>
       <c r="I62" t="n">
-        <v>4562.476</v>
+        <v>4796.3335</v>
       </c>
       <c r="J62" t="n">
         <v>6578.0835</v>
       </c>
       <c r="K62" t="n">
-        <v>4562.476</v>
+        <v>4796.3335</v>
       </c>
       <c r="L62" t="n">
         <v>6578.0835</v>
       </c>
       <c r="M62" t="n">
-        <v>-3938.476</v>
+        <v>-4172.3335</v>
       </c>
       <c r="N62" t="n">
         <v>-7826.0835</v>
@@ -3827,22 +3827,22 @@
         <v>27781</v>
       </c>
       <c r="H65" t="n">
-        <v>5295.4243</v>
+        <v>5390.25</v>
       </c>
       <c r="I65" t="n">
-        <v>4562.476</v>
+        <v>4796.3335</v>
       </c>
       <c r="J65" t="n">
         <v>6578.0835</v>
       </c>
       <c r="K65" t="n">
-        <v>22812.38</v>
+        <v>23981.6675</v>
       </c>
       <c r="L65" t="n">
         <v>32890.4175</v>
       </c>
       <c r="M65" t="n">
-        <v>-19692.38</v>
+        <v>-20861.6675</v>
       </c>
       <c r="N65" t="n">
         <v>-39130.4175</v>
@@ -4366,22 +4366,22 @@
         <v>12602</v>
       </c>
       <c r="H76" t="n">
-        <v>2999.5</v>
+        <v>2999</v>
       </c>
       <c r="I76" t="n">
-        <v>2999.5</v>
+        <v>2999</v>
       </c>
       <c r="J76" t="n">
         <v>0</v>
       </c>
       <c r="K76" t="n">
-        <v>2999.5</v>
+        <v>2999</v>
       </c>
       <c r="L76" t="n">
         <v>0</v>
       </c>
       <c r="M76" t="n">
-        <v>-2684.5</v>
+        <v>-2684</v>
       </c>
     </row>
     <row r="77">
@@ -4513,22 +4513,22 @@
         <v>12602</v>
       </c>
       <c r="H79" t="n">
-        <v>2999.5</v>
+        <v>2999</v>
       </c>
       <c r="I79" t="n">
-        <v>2999.5</v>
+        <v>2999</v>
       </c>
       <c r="J79" t="n">
         <v>0</v>
       </c>
       <c r="K79" t="n">
-        <v>2999.5</v>
+        <v>2999</v>
       </c>
       <c r="L79" t="n">
         <v>0</v>
       </c>
       <c r="M79" t="n">
-        <v>-1907.5</v>
+        <v>-1907</v>
       </c>
     </row>
     <row r="80">
@@ -5309,22 +5309,22 @@
         <v>18200</v>
       </c>
       <c r="H95" t="n">
-        <v>63913.668</v>
+        <v>67396.39999999999</v>
       </c>
       <c r="I95" t="n">
         <v>0</v>
       </c>
       <c r="J95" t="n">
-        <v>63913.668</v>
+        <v>67396.39999999999</v>
       </c>
       <c r="K95" t="n">
         <v>0</v>
       </c>
       <c r="L95" t="n">
-        <v>63913.668</v>
+        <v>67396.39999999999</v>
       </c>
       <c r="N95" t="n">
-        <v>-69405.66800000001</v>
+        <v>-72888.39999999999</v>
       </c>
     </row>
     <row r="96">
@@ -5713,25 +5713,25 @@
         <v>19909</v>
       </c>
       <c r="H103" t="n">
-        <v>784.1698</v>
+        <v>725.76</v>
       </c>
       <c r="I103" t="n">
-        <v>781.7895</v>
+        <v>672.3143</v>
       </c>
       <c r="J103" t="n">
-        <v>790.2</v>
+        <v>850.4666999999999</v>
       </c>
       <c r="K103" t="n">
-        <v>2345.3685</v>
+        <v>2016.9429</v>
       </c>
       <c r="L103" t="n">
-        <v>2370.6</v>
+        <v>2551.4001</v>
       </c>
       <c r="M103" t="n">
-        <v>-1759.3685</v>
+        <v>-1430.9429</v>
       </c>
       <c r="N103" t="n">
-        <v>-3542.6</v>
+        <v>-3723.4001</v>
       </c>
     </row>
     <row r="104">
@@ -5817,22 +5817,22 @@
         <v>18668</v>
       </c>
       <c r="H105" t="n">
-        <v>67417.5</v>
+        <v>63934</v>
       </c>
       <c r="I105" t="n">
         <v>0</v>
       </c>
       <c r="J105" t="n">
-        <v>67417.5</v>
+        <v>63934</v>
       </c>
       <c r="K105" t="n">
         <v>0</v>
       </c>
       <c r="L105" t="n">
-        <v>67417.5</v>
+        <v>63934</v>
       </c>
       <c r="N105" t="n">
-        <v>-74405.5</v>
+        <v>-70922</v>
       </c>
     </row>
     <row r="106">
@@ -6215,22 +6215,22 @@
         <v>27775</v>
       </c>
       <c r="H113" t="n">
-        <v>2040</v>
+        <v>2016.8422</v>
       </c>
       <c r="I113" t="n">
-        <v>2040</v>
+        <v>2016.8422</v>
       </c>
       <c r="J113" t="n">
         <v>0</v>
       </c>
       <c r="K113" t="n">
-        <v>2040</v>
+        <v>2016.8422</v>
       </c>
       <c r="L113" t="n">
         <v>0</v>
       </c>
       <c r="M113" t="n">
-        <v>1214</v>
+        <v>1237.1578</v>
       </c>
     </row>
     <row r="114">
@@ -7143,25 +7143,25 @@
         <v>44049</v>
       </c>
       <c r="H132" t="n">
-        <v>733.2857</v>
+        <v>831.7222</v>
       </c>
       <c r="I132" t="n">
-        <v>558.9231</v>
+        <v>623.1875</v>
       </c>
       <c r="J132" t="n">
-        <v>3000</v>
+        <v>2500</v>
       </c>
       <c r="K132" t="n">
-        <v>1676.7693</v>
+        <v>1869.5625</v>
       </c>
       <c r="L132" t="n">
-        <v>9000</v>
+        <v>7500</v>
       </c>
       <c r="M132" t="n">
-        <v>853.2307000000001</v>
+        <v>660.4375</v>
       </c>
       <c r="N132" t="n">
-        <v>-14060</v>
+        <v>-12560</v>
       </c>
     </row>
     <row r="133">
@@ -7443,25 +7443,25 @@
         <v>44169</v>
       </c>
       <c r="H138" t="n">
-        <v>6470.2856</v>
+        <v>6277.0454</v>
       </c>
       <c r="I138" t="n">
-        <v>6028.8184</v>
+        <v>6001.5454</v>
       </c>
       <c r="J138" t="n">
-        <v>6955.9</v>
+        <v>6552.5454</v>
       </c>
       <c r="K138" t="n">
-        <v>18086.4552</v>
+        <v>18004.6362</v>
       </c>
       <c r="L138" t="n">
-        <v>20867.7</v>
+        <v>19657.6362</v>
       </c>
       <c r="M138" t="n">
-        <v>-12946.4552</v>
+        <v>-12864.6362</v>
       </c>
       <c r="N138" t="n">
-        <v>-31147.7</v>
+        <v>-29937.6362</v>
       </c>
     </row>
     <row r="139">
@@ -7590,22 +7590,22 @@
         <v>44161</v>
       </c>
       <c r="H141" t="n">
-        <v>8321.111000000001</v>
+        <v>7989</v>
       </c>
       <c r="I141" t="n">
-        <v>8111.25</v>
+        <v>7765.5557</v>
       </c>
       <c r="J141" t="n">
         <v>10000</v>
       </c>
       <c r="K141" t="n">
-        <v>24333.75</v>
+        <v>23296.6671</v>
       </c>
       <c r="L141" t="n">
         <v>30000</v>
       </c>
       <c r="M141" t="n">
-        <v>-19153.75</v>
+        <v>-18116.6671</v>
       </c>
       <c r="N141" t="n">
         <v>-40360</v>
@@ -7731,22 +7731,22 @@
         <v>27713</v>
       </c>
       <c r="H2" t="n">
-        <v>837.2857</v>
+        <v>785.06665</v>
       </c>
       <c r="I2" t="n">
-        <v>840.53845</v>
+        <v>784.3570999999999</v>
       </c>
       <c r="J2" t="n">
         <v>795</v>
       </c>
       <c r="K2" t="n">
-        <v>840.53845</v>
+        <v>784.3570999999999</v>
       </c>
       <c r="L2" t="n">
         <v>795</v>
       </c>
       <c r="M2" t="n">
-        <v>-727.53845</v>
+        <v>-671.3570999999999</v>
       </c>
       <c r="N2" t="n">
         <v>-1021</v>
@@ -7875,22 +7875,22 @@
         <v>5091</v>
       </c>
       <c r="H5" t="n">
-        <v>400</v>
+        <v>361</v>
       </c>
       <c r="I5" t="n">
-        <v>400</v>
+        <v>361</v>
       </c>
       <c r="J5" t="n">
         <v>0</v>
       </c>
       <c r="K5" t="n">
-        <v>400</v>
+        <v>361</v>
       </c>
       <c r="L5" t="n">
         <v>0</v>
       </c>
       <c r="M5" t="n">
-        <v>-288</v>
+        <v>-249</v>
       </c>
     </row>
     <row r="6">
@@ -8815,22 +8815,22 @@
         <v>18363</v>
       </c>
       <c r="H24" t="n">
-        <v>355</v>
+        <v>20177.5</v>
       </c>
       <c r="I24" t="n">
         <v>0</v>
       </c>
       <c r="J24" t="n">
-        <v>355</v>
+        <v>20177.5</v>
       </c>
       <c r="K24" t="n">
         <v>0</v>
       </c>
       <c r="L24" t="n">
-        <v>355</v>
+        <v>20177.5</v>
       </c>
       <c r="N24" t="n">
-        <v>-1103</v>
+        <v>-20925.5</v>
       </c>
     </row>
     <row r="25">
@@ -9063,25 +9063,25 @@
         <v>3557</v>
       </c>
       <c r="H29" t="n">
-        <v>11275.333</v>
+        <v>11203.111</v>
       </c>
       <c r="I29" t="n">
-        <v>6289</v>
+        <v>11578</v>
       </c>
       <c r="J29" t="n">
-        <v>12700</v>
+        <v>11156.25</v>
       </c>
       <c r="K29" t="n">
-        <v>6289</v>
+        <v>11578</v>
       </c>
       <c r="L29" t="n">
-        <v>12700</v>
+        <v>11156.25</v>
       </c>
       <c r="M29" t="n">
-        <v>-5981</v>
+        <v>-11270</v>
       </c>
       <c r="N29" t="n">
-        <v>-13316</v>
+        <v>-11772.25</v>
       </c>
     </row>
     <row r="30">
@@ -9115,25 +9115,25 @@
         <v>2712</v>
       </c>
       <c r="H30" t="n">
-        <v>10002</v>
+        <v>4677.25</v>
       </c>
       <c r="I30" t="n">
-        <v>6004.5</v>
+        <v>1736.3334</v>
       </c>
       <c r="J30" t="n">
-        <v>13999.5</v>
+        <v>13500</v>
       </c>
       <c r="K30" t="n">
-        <v>6004.5</v>
+        <v>1736.3334</v>
       </c>
       <c r="L30" t="n">
-        <v>13999.5</v>
+        <v>13500</v>
       </c>
       <c r="M30" t="n">
-        <v>-5854.5</v>
+        <v>-1586.3334</v>
       </c>
       <c r="N30" t="n">
-        <v>-14299.5</v>
+        <v>-13800</v>
       </c>
     </row>
     <row r="31">
@@ -9219,25 +9219,25 @@
         <v>44147</v>
       </c>
       <c r="H32" t="n">
-        <v>1952840.8</v>
+        <v>2510716.2</v>
       </c>
       <c r="I32" t="n">
-        <v>491409.06</v>
+        <v>640912.0600000001</v>
       </c>
       <c r="J32" t="n">
-        <v>9259999</v>
+        <v>11111816</v>
       </c>
       <c r="K32" t="n">
-        <v>491409.06</v>
+        <v>640912.0600000001</v>
       </c>
       <c r="L32" t="n">
-        <v>9259999</v>
+        <v>11111816</v>
       </c>
       <c r="M32" t="n">
-        <v>-491122.06</v>
+        <v>-640625.0600000001</v>
       </c>
       <c r="N32" t="n">
-        <v>-9260573</v>
+        <v>-11112390</v>
       </c>
     </row>
     <row r="33">
@@ -9320,22 +9320,22 @@
         <v>2753</v>
       </c>
       <c r="H34" t="n">
-        <v>75368.14999999999</v>
+        <v>88380.53</v>
       </c>
       <c r="I34" t="n">
-        <v>53019.105</v>
+        <v>62654.312</v>
       </c>
       <c r="J34" t="n">
         <v>500000</v>
       </c>
       <c r="K34" t="n">
-        <v>53019.105</v>
+        <v>62654.312</v>
       </c>
       <c r="L34" t="n">
         <v>500000</v>
       </c>
       <c r="M34" t="n">
-        <v>-52748.105</v>
+        <v>-62383.312</v>
       </c>
       <c r="N34" t="n">
         <v>-500542</v>
@@ -9966,25 +9966,25 @@
         <v>3622</v>
       </c>
       <c r="H47" t="n">
-        <v>30000</v>
+        <v>34983.332</v>
       </c>
       <c r="I47" t="n">
         <v>15000</v>
       </c>
       <c r="J47" t="n">
-        <v>45000</v>
+        <v>44975</v>
       </c>
       <c r="K47" t="n">
         <v>15000</v>
       </c>
       <c r="L47" t="n">
-        <v>45000</v>
+        <v>44975</v>
       </c>
       <c r="M47" t="n">
         <v>-14275</v>
       </c>
       <c r="N47" t="n">
-        <v>-46450</v>
+        <v>-46425</v>
       </c>
     </row>
     <row r="48">
@@ -10110,25 +10110,25 @@
         <v>27657</v>
       </c>
       <c r="H50" t="n">
-        <v>5088.778</v>
+        <v>665.44446</v>
       </c>
       <c r="I50" t="n">
-        <v>8420</v>
+        <v>525</v>
       </c>
       <c r="J50" t="n">
-        <v>924.75</v>
+        <v>777.8</v>
       </c>
       <c r="K50" t="n">
-        <v>8420</v>
+        <v>525</v>
       </c>
       <c r="L50" t="n">
-        <v>924.75</v>
+        <v>777.8</v>
       </c>
       <c r="M50" t="n">
-        <v>-7706</v>
+        <v>189</v>
       </c>
       <c r="N50" t="n">
-        <v>-2352.75</v>
+        <v>-2205.8</v>
       </c>
     </row>
     <row r="51">
@@ -10637,22 +10637,22 @@
         <v>43999</v>
       </c>
       <c r="H61" t="n">
-        <v>2727.7551</v>
+        <v>2729.1836</v>
       </c>
       <c r="I61" t="n">
-        <v>1562.7742</v>
+        <v>1565.0322</v>
       </c>
       <c r="J61" t="n">
         <v>4734.1113</v>
       </c>
       <c r="K61" t="n">
-        <v>1562.7742</v>
+        <v>1565.0322</v>
       </c>
       <c r="L61" t="n">
         <v>4734.1113</v>
       </c>
       <c r="M61" t="n">
-        <v>-1350.7742</v>
+        <v>-1353.0322</v>
       </c>
       <c r="N61" t="n">
         <v>-5158.1113</v>
@@ -10738,22 +10738,25 @@
         <v>12528</v>
       </c>
       <c r="H63" t="n">
-        <v>1635</v>
+        <v>3567.2222</v>
       </c>
       <c r="I63" t="n">
-        <v>1635</v>
+        <v>2021</v>
       </c>
       <c r="J63" t="n">
-        <v>0</v>
+        <v>5500</v>
       </c>
       <c r="K63" t="n">
-        <v>1635</v>
+        <v>2021</v>
       </c>
       <c r="L63" t="n">
-        <v>0</v>
+        <v>5500</v>
       </c>
       <c r="M63" t="n">
-        <v>-949</v>
+        <v>-1335</v>
+      </c>
+      <c r="N63" t="n">
+        <v>-6872</v>
       </c>
     </row>
     <row r="64">
@@ -10882,22 +10885,25 @@
         <v>12528</v>
       </c>
       <c r="H66" t="n">
-        <v>1635</v>
+        <v>3567.2222</v>
       </c>
       <c r="I66" t="n">
-        <v>1635</v>
+        <v>2021</v>
       </c>
       <c r="J66" t="n">
-        <v>0</v>
+        <v>5500</v>
       </c>
       <c r="K66" t="n">
-        <v>8175</v>
+        <v>10105</v>
       </c>
       <c r="L66" t="n">
-        <v>0</v>
+        <v>27500</v>
       </c>
       <c r="M66" t="n">
-        <v>-4743</v>
+        <v>-6673</v>
+      </c>
+      <c r="N66" t="n">
+        <v>-34364</v>
       </c>
     </row>
     <row r="67">
@@ -12518,22 +12524,22 @@
         <v>18363</v>
       </c>
       <c r="H100" t="n">
-        <v>355</v>
+        <v>20177.5</v>
       </c>
       <c r="I100" t="n">
         <v>0</v>
       </c>
       <c r="J100" t="n">
-        <v>355</v>
+        <v>20177.5</v>
       </c>
       <c r="K100" t="n">
         <v>0</v>
       </c>
       <c r="L100" t="n">
-        <v>355</v>
+        <v>20177.5</v>
       </c>
       <c r="N100" t="n">
-        <v>-2519</v>
+        <v>-22341.5</v>
       </c>
     </row>
     <row r="101">
@@ -12993,25 +12999,25 @@
         <v>27708</v>
       </c>
       <c r="H110" t="n">
-        <v>62501744</v>
+        <v>58825356</v>
       </c>
       <c r="I110" t="n">
-        <v>527.4</v>
+        <v>657.4</v>
       </c>
       <c r="J110" t="n">
-        <v>90911390</v>
+        <v>83335650</v>
       </c>
       <c r="K110" t="n">
-        <v>527.4</v>
+        <v>657.4</v>
       </c>
       <c r="L110" t="n">
-        <v>90911390</v>
+        <v>83335650</v>
       </c>
       <c r="M110" t="n">
-        <v>1517.6</v>
+        <v>1387.6</v>
       </c>
       <c r="N110" t="n">
-        <v>-90915480</v>
+        <v>-83339740</v>
       </c>
     </row>
     <row r="111">
@@ -13284,22 +13290,22 @@
         <v>27713</v>
       </c>
       <c r="H116" t="n">
-        <v>837.2857</v>
+        <v>785.06665</v>
       </c>
       <c r="I116" t="n">
-        <v>840.53845</v>
+        <v>784.3570999999999</v>
       </c>
       <c r="J116" t="n">
         <v>795</v>
       </c>
       <c r="K116" t="n">
-        <v>840.53845</v>
+        <v>784.3570999999999</v>
       </c>
       <c r="L116" t="n">
         <v>795</v>
       </c>
       <c r="M116" t="n">
-        <v>1453.46155</v>
+        <v>1509.6429</v>
       </c>
       <c r="N116" t="n">
         <v>-5383</v>
@@ -14065,22 +14071,22 @@
         <v>43997</v>
       </c>
       <c r="H132" t="n">
-        <v>6229.8335</v>
+        <v>6008.88</v>
       </c>
       <c r="I132" t="n">
-        <v>6547.7144</v>
+        <v>6282.1816</v>
       </c>
       <c r="J132" t="n">
         <v>4004.6667</v>
       </c>
       <c r="K132" t="n">
-        <v>19643.1432</v>
+        <v>18846.5448</v>
       </c>
       <c r="L132" t="n">
         <v>12014.0001</v>
       </c>
       <c r="M132" t="n">
-        <v>-17113.1432</v>
+        <v>-16316.5448</v>
       </c>
       <c r="N132" t="n">
         <v>-17074.0001</v>
@@ -14261,22 +14267,22 @@
         <v>43999</v>
       </c>
       <c r="H136" t="n">
-        <v>2727.7551</v>
+        <v>2729.1836</v>
       </c>
       <c r="I136" t="n">
-        <v>1562.7742</v>
+        <v>1565.0322</v>
       </c>
       <c r="J136" t="n">
         <v>4734.1113</v>
       </c>
       <c r="K136" t="n">
-        <v>4688.3226</v>
+        <v>4695.096600000001</v>
       </c>
       <c r="L136" t="n">
         <v>14202.3339</v>
       </c>
       <c r="M136" t="n">
-        <v>-2138.3226</v>
+        <v>-2145.096600000001</v>
       </c>
       <c r="N136" t="n">
         <v>-19302.3339</v>
@@ -14687,22 +14693,22 @@
         <v>27713</v>
       </c>
       <c r="H3" t="n">
-        <v>837.2857</v>
+        <v>785.06665</v>
       </c>
       <c r="I3" t="n">
-        <v>840.53845</v>
+        <v>784.3570999999999</v>
       </c>
       <c r="J3" t="n">
         <v>795</v>
       </c>
       <c r="K3" t="n">
-        <v>840.53845</v>
+        <v>784.3570999999999</v>
       </c>
       <c r="L3" t="n">
         <v>795</v>
       </c>
       <c r="M3" t="n">
-        <v>-726.53845</v>
+        <v>-670.3570999999999</v>
       </c>
       <c r="N3" t="n">
         <v>-1023</v>
@@ -14739,22 +14745,22 @@
         <v>5091</v>
       </c>
       <c r="H4" t="n">
-        <v>400</v>
+        <v>361</v>
       </c>
       <c r="I4" t="n">
-        <v>400</v>
+        <v>361</v>
       </c>
       <c r="J4" t="n">
         <v>0</v>
       </c>
       <c r="K4" t="n">
-        <v>400</v>
+        <v>361</v>
       </c>
       <c r="L4" t="n">
         <v>0</v>
       </c>
       <c r="M4" t="n">
-        <v>-285</v>
+        <v>-246</v>
       </c>
     </row>
     <row r="5">
@@ -15180,22 +15186,22 @@
         <v>27127</v>
       </c>
       <c r="H13" t="n">
-        <v>78482.60000000001</v>
+        <v>82067.164</v>
       </c>
       <c r="I13" t="n">
         <v>0</v>
       </c>
       <c r="J13" t="n">
-        <v>78482.60000000001</v>
+        <v>82067.164</v>
       </c>
       <c r="K13" t="n">
         <v>0</v>
       </c>
       <c r="L13" t="n">
-        <v>78482.60000000001</v>
+        <v>82067.164</v>
       </c>
       <c r="N13" t="n">
-        <v>-78818.60000000001</v>
+        <v>-82403.164</v>
       </c>
     </row>
     <row r="14">
@@ -15229,22 +15235,22 @@
         <v>2342</v>
       </c>
       <c r="H14" t="n">
-        <v>724.75</v>
+        <v>574.75</v>
       </c>
       <c r="I14" t="n">
         <v>0</v>
       </c>
       <c r="J14" t="n">
-        <v>724.75</v>
+        <v>574.75</v>
       </c>
       <c r="K14" t="n">
         <v>0</v>
       </c>
       <c r="L14" t="n">
-        <v>724.75</v>
+        <v>574.75</v>
       </c>
       <c r="N14" t="n">
-        <v>-1068.75</v>
+        <v>-918.75</v>
       </c>
     </row>
     <row r="15">
@@ -15609,25 +15615,25 @@
         <v>5092</v>
       </c>
       <c r="H22" t="n">
-        <v>18520692</v>
+        <v>18870130</v>
       </c>
       <c r="I22" t="n">
-        <v>20409532</v>
+        <v>20001344</v>
       </c>
       <c r="J22" t="n">
-        <v>10064</v>
+        <v>16566.666</v>
       </c>
       <c r="K22" t="n">
-        <v>20409532</v>
+        <v>20001344</v>
       </c>
       <c r="L22" t="n">
-        <v>10064</v>
+        <v>16566.666</v>
       </c>
       <c r="M22" t="n">
-        <v>-20409359</v>
+        <v>-20001171</v>
       </c>
       <c r="N22" t="n">
-        <v>-10410</v>
+        <v>-16912.666</v>
       </c>
     </row>
     <row r="23">
@@ -18452,22 +18458,22 @@
         <v>42300</v>
       </c>
       <c r="H81" t="n">
-        <v>73098.8</v>
+        <v>89373.5</v>
       </c>
       <c r="I81" t="n">
         <v>0</v>
       </c>
       <c r="J81" t="n">
-        <v>73098.8</v>
+        <v>89373.5</v>
       </c>
       <c r="K81" t="n">
         <v>0</v>
       </c>
       <c r="L81" t="n">
-        <v>73098.8</v>
+        <v>89373.5</v>
       </c>
       <c r="N81" t="n">
-        <v>-75220.8</v>
+        <v>-91495.5</v>
       </c>
     </row>
     <row r="82">
@@ -18501,23 +18507,26 @@
         <v>11877</v>
       </c>
       <c r="H82" t="n">
-        <v>44975</v>
+        <v>46650</v>
       </c>
       <c r="I82" t="n">
         <v>44975</v>
       </c>
       <c r="J82" t="n">
-        <v>0</v>
+        <v>50000</v>
       </c>
       <c r="K82" t="n">
         <v>44975</v>
       </c>
       <c r="L82" t="n">
-        <v>0</v>
+        <v>50000</v>
       </c>
       <c r="M82" t="n">
         <v>-44592</v>
       </c>
+      <c r="N82" t="n">
+        <v>-50766</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -18602,22 +18611,22 @@
         <v>42300</v>
       </c>
       <c r="H84" t="n">
-        <v>73098.8</v>
+        <v>89373.5</v>
       </c>
       <c r="I84" t="n">
         <v>0</v>
       </c>
       <c r="J84" t="n">
-        <v>73098.8</v>
+        <v>89373.5</v>
       </c>
       <c r="K84" t="n">
         <v>0</v>
       </c>
       <c r="L84" t="n">
-        <v>219296.4</v>
+        <v>268120.5</v>
       </c>
       <c r="N84" t="n">
-        <v>-229904.4</v>
+        <v>-278728.5</v>
       </c>
     </row>
     <row r="85">
@@ -18651,23 +18660,26 @@
         <v>11877</v>
       </c>
       <c r="H85" t="n">
-        <v>44975</v>
+        <v>46650</v>
       </c>
       <c r="I85" t="n">
         <v>44975</v>
       </c>
       <c r="J85" t="n">
-        <v>0</v>
+        <v>50000</v>
       </c>
       <c r="K85" t="n">
         <v>44975</v>
       </c>
       <c r="L85" t="n">
-        <v>0</v>
+        <v>50000</v>
       </c>
       <c r="M85" t="n">
         <v>-43649</v>
       </c>
+      <c r="N85" t="n">
+        <v>-52652</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -18700,25 +18712,25 @@
         <v>12526</v>
       </c>
       <c r="H86" t="n">
-        <v>2172.5</v>
+        <v>3135.2222</v>
       </c>
       <c r="I86" t="n">
-        <v>1403.6666</v>
+        <v>1872.5</v>
       </c>
       <c r="J86" t="n">
-        <v>3556.4</v>
+        <v>5660.6665</v>
       </c>
       <c r="K86" t="n">
-        <v>1403.6666</v>
+        <v>1872.5</v>
       </c>
       <c r="L86" t="n">
-        <v>3556.4</v>
+        <v>5660.6665</v>
       </c>
       <c r="M86" t="n">
-        <v>-280.6666</v>
+        <v>-749.5</v>
       </c>
       <c r="N86" t="n">
-        <v>-5802.4</v>
+        <v>-7906.6665</v>
       </c>
     </row>
     <row r="87">
@@ -18850,25 +18862,25 @@
         <v>12526</v>
       </c>
       <c r="H89" t="n">
-        <v>2172.5</v>
+        <v>3135.2222</v>
       </c>
       <c r="I89" t="n">
-        <v>1403.6666</v>
+        <v>1872.5</v>
       </c>
       <c r="J89" t="n">
-        <v>3556.4</v>
+        <v>5660.6665</v>
       </c>
       <c r="K89" t="n">
-        <v>7018.333000000001</v>
+        <v>9362.5</v>
       </c>
       <c r="L89" t="n">
-        <v>17782</v>
+        <v>28303.3325</v>
       </c>
       <c r="M89" t="n">
-        <v>-1402.333000000001</v>
+        <v>-3746.5</v>
       </c>
       <c r="N89" t="n">
-        <v>-29014</v>
+        <v>-39535.3325</v>
       </c>
     </row>
     <row r="90">
@@ -19245,23 +19257,26 @@
         <v>19518</v>
       </c>
       <c r="H97" t="n">
-        <v>3539.25</v>
+        <v>3382.4443</v>
       </c>
       <c r="I97" t="n">
         <v>3539.25</v>
       </c>
       <c r="J97" t="n">
-        <v>0</v>
+        <v>2128</v>
       </c>
       <c r="K97" t="n">
         <v>3539.25</v>
       </c>
       <c r="L97" t="n">
-        <v>0</v>
+        <v>2128</v>
       </c>
       <c r="M97" t="n">
         <v>-2548.25</v>
       </c>
+      <c r="N97" t="n">
+        <v>-4110</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -19343,22 +19358,22 @@
         <v>19943</v>
       </c>
       <c r="H99" t="n">
-        <v>3054.5715</v>
+        <v>2952</v>
       </c>
       <c r="I99" t="n">
-        <v>2776.3684</v>
+        <v>2677.45</v>
       </c>
       <c r="J99" t="n">
         <v>5697.5</v>
       </c>
       <c r="K99" t="n">
-        <v>2776.3684</v>
+        <v>2677.45</v>
       </c>
       <c r="L99" t="n">
         <v>5697.5</v>
       </c>
       <c r="M99" t="n">
-        <v>-1278.3684</v>
+        <v>-1179.45</v>
       </c>
       <c r="N99" t="n">
         <v>-8693.5</v>
@@ -19631,22 +19646,22 @@
         <v>19947</v>
       </c>
       <c r="H105" t="n">
-        <v>2146.75</v>
+        <v>2004.6666</v>
       </c>
       <c r="I105" t="n">
-        <v>1978.2727</v>
+        <v>1862.1428</v>
       </c>
       <c r="J105" t="n">
         <v>4000</v>
       </c>
       <c r="K105" t="n">
-        <v>1978.2727</v>
+        <v>1862.1428</v>
       </c>
       <c r="L105" t="n">
         <v>4000</v>
       </c>
       <c r="M105" t="n">
-        <v>-231.2727</v>
+        <v>-115.1428000000001</v>
       </c>
       <c r="N105" t="n">
         <v>-7494</v>
@@ -19732,25 +19747,25 @@
         <v>27706</v>
       </c>
       <c r="H107" t="n">
-        <v>943.35297</v>
+        <v>1004.3</v>
       </c>
       <c r="I107" t="n">
-        <v>862.2963</v>
+        <v>861.88</v>
       </c>
       <c r="J107" t="n">
-        <v>1256</v>
+        <v>1716.4</v>
       </c>
       <c r="K107" t="n">
-        <v>862.2963</v>
+        <v>861.88</v>
       </c>
       <c r="L107" t="n">
-        <v>1256</v>
+        <v>1716.4</v>
       </c>
       <c r="M107" t="n">
-        <v>1057.7037</v>
+        <v>1058.12</v>
       </c>
       <c r="N107" t="n">
-        <v>-5096</v>
+        <v>-5556.4</v>
       </c>
     </row>
     <row r="108">
@@ -21019,22 +21034,22 @@
         <v>43998</v>
       </c>
       <c r="H134" t="n">
-        <v>1668821.4</v>
+        <v>1628116</v>
       </c>
       <c r="I134" t="n">
-        <v>1756456.6</v>
+        <v>1711416.8</v>
       </c>
       <c r="J134" t="n">
         <v>3750</v>
       </c>
       <c r="K134" t="n">
-        <v>5269369.800000001</v>
+        <v>5134250.4</v>
       </c>
       <c r="L134" t="n">
         <v>11250</v>
       </c>
       <c r="M134" t="n">
-        <v>-5266834.800000001</v>
+        <v>-5131715.4</v>
       </c>
       <c r="N134" t="n">
         <v>-16320</v>
@@ -21748,22 +21763,22 @@
         <v>5361</v>
       </c>
       <c r="H7" t="n">
-        <v>87</v>
+        <v>82.70587999999999</v>
       </c>
       <c r="I7" t="n">
-        <v>91.46666999999999</v>
+        <v>86.625</v>
       </c>
       <c r="J7" t="n">
         <v>20</v>
       </c>
       <c r="K7" t="n">
-        <v>91.46666999999999</v>
+        <v>86.625</v>
       </c>
       <c r="L7" t="n">
         <v>20</v>
       </c>
       <c r="M7" t="n">
-        <v>21.53333000000001</v>
+        <v>26.375</v>
       </c>
       <c r="N7" t="n">
         <v>-246</v>
@@ -22183,22 +22198,22 @@
         <v>27691</v>
       </c>
       <c r="H16" t="n">
-        <v>2673.3635</v>
+        <v>2670.4546</v>
       </c>
       <c r="I16" t="n">
-        <v>1270.7142</v>
+        <v>1261.5714</v>
       </c>
       <c r="J16" t="n">
         <v>3327.9333</v>
       </c>
       <c r="K16" t="n">
-        <v>1270.7142</v>
+        <v>1261.5714</v>
       </c>
       <c r="L16" t="n">
         <v>3327.9333</v>
       </c>
       <c r="M16" t="n">
-        <v>-983.7141999999999</v>
+        <v>-974.5714</v>
       </c>
       <c r="N16" t="n">
         <v>-3901.9333</v>
@@ -22327,22 +22342,22 @@
         <v>2233</v>
       </c>
       <c r="H19" t="n">
-        <v>1398.2222</v>
+        <v>1268.4</v>
       </c>
       <c r="I19" t="n">
-        <v>1398.2222</v>
+        <v>1268.4</v>
       </c>
       <c r="J19" t="n">
         <v>0</v>
       </c>
       <c r="K19" t="n">
-        <v>1398.2222</v>
+        <v>1268.4</v>
       </c>
       <c r="L19" t="n">
         <v>0</v>
       </c>
       <c r="M19" t="n">
-        <v>-1228.2222</v>
+        <v>-1098.4</v>
       </c>
     </row>
     <row r="20">
@@ -22572,22 +22587,22 @@
         <v>2233</v>
       </c>
       <c r="H24" t="n">
-        <v>1398.2222</v>
+        <v>1268.4</v>
       </c>
       <c r="I24" t="n">
-        <v>1398.2222</v>
+        <v>1268.4</v>
       </c>
       <c r="J24" t="n">
         <v>0</v>
       </c>
       <c r="K24" t="n">
-        <v>1398.2222</v>
+        <v>1268.4</v>
       </c>
       <c r="L24" t="n">
         <v>0</v>
       </c>
       <c r="M24" t="n">
-        <v>-1228.2222</v>
+        <v>-1098.4</v>
       </c>
     </row>
     <row r="25">
@@ -23181,22 +23196,22 @@
         <v>1845</v>
       </c>
       <c r="H36" t="n">
-        <v>34310.92</v>
+        <v>33080.152</v>
       </c>
       <c r="I36" t="n">
-        <v>32170.166</v>
+        <v>30836.834</v>
       </c>
       <c r="J36" t="n">
         <v>60000</v>
       </c>
       <c r="K36" t="n">
-        <v>32170.166</v>
+        <v>30836.834</v>
       </c>
       <c r="L36" t="n">
         <v>60000</v>
       </c>
       <c r="M36" t="n">
-        <v>-31782.166</v>
+        <v>-30448.834</v>
       </c>
       <c r="N36" t="n">
         <v>-60776</v>
@@ -23377,22 +23392,22 @@
         <v>1845</v>
       </c>
       <c r="H40" t="n">
-        <v>34310.92</v>
+        <v>33080.152</v>
       </c>
       <c r="I40" t="n">
-        <v>32170.166</v>
+        <v>30836.834</v>
       </c>
       <c r="J40" t="n">
         <v>60000</v>
       </c>
       <c r="K40" t="n">
-        <v>32170.166</v>
+        <v>30836.834</v>
       </c>
       <c r="L40" t="n">
         <v>60000</v>
       </c>
       <c r="M40" t="n">
-        <v>-32010.166</v>
+        <v>-30676.834</v>
       </c>
       <c r="N40" t="n">
         <v>-60320</v>
@@ -24100,22 +24115,22 @@
         <v>1855</v>
       </c>
       <c r="H55" t="n">
-        <v>8166.6665</v>
+        <v>7833.3335</v>
       </c>
       <c r="I55" t="n">
-        <v>8166.6665</v>
+        <v>7833.3335</v>
       </c>
       <c r="J55" t="n">
         <v>0</v>
       </c>
       <c r="K55" t="n">
-        <v>8166.6665</v>
+        <v>7833.3335</v>
       </c>
       <c r="L55" t="n">
         <v>0</v>
       </c>
       <c r="M55" t="n">
-        <v>-7851.6665</v>
+        <v>-7518.3335</v>
       </c>
     </row>
     <row r="56">
@@ -24244,25 +24259,25 @@
         <v>44021</v>
       </c>
       <c r="H58" t="n">
-        <v>6503.5625</v>
+        <v>6243.4116</v>
       </c>
       <c r="I58" t="n">
-        <v>6325.5356</v>
+        <v>6176.793</v>
       </c>
       <c r="J58" t="n">
-        <v>7749.75</v>
+        <v>6629.8</v>
       </c>
       <c r="K58" t="n">
-        <v>6325.5356</v>
+        <v>6176.793</v>
       </c>
       <c r="L58" t="n">
-        <v>7749.75</v>
+        <v>6629.8</v>
       </c>
       <c r="M58" t="n">
-        <v>-6122.5356</v>
+        <v>-5973.793</v>
       </c>
       <c r="N58" t="n">
-        <v>-8155.75</v>
+        <v>-7035.8</v>
       </c>
     </row>
     <row r="59">
@@ -25598,25 +25613,25 @@
         <v>12584</v>
       </c>
       <c r="H86" t="n">
-        <v>21799.8</v>
+        <v>20142.715</v>
       </c>
       <c r="I86" t="n">
-        <v>24999</v>
+        <v>18499.5</v>
       </c>
       <c r="J86" t="n">
-        <v>21000</v>
+        <v>20800</v>
       </c>
       <c r="K86" t="n">
-        <v>24999</v>
+        <v>18499.5</v>
       </c>
       <c r="L86" t="n">
-        <v>21000</v>
+        <v>20800</v>
       </c>
       <c r="M86" t="n">
-        <v>-23876</v>
+        <v>-17376.5</v>
       </c>
       <c r="N86" t="n">
-        <v>-23246</v>
+        <v>-23046</v>
       </c>
     </row>
     <row r="87">
@@ -25745,25 +25760,25 @@
         <v>12584</v>
       </c>
       <c r="H89" t="n">
-        <v>21799.8</v>
+        <v>20142.715</v>
       </c>
       <c r="I89" t="n">
-        <v>24999</v>
+        <v>18499.5</v>
       </c>
       <c r="J89" t="n">
-        <v>21000</v>
+        <v>20800</v>
       </c>
       <c r="K89" t="n">
-        <v>124995</v>
+        <v>92497.5</v>
       </c>
       <c r="L89" t="n">
-        <v>105000</v>
+        <v>104000</v>
       </c>
       <c r="M89" t="n">
-        <v>-119379</v>
+        <v>-86881.5</v>
       </c>
       <c r="N89" t="n">
-        <v>-116232</v>
+        <v>-115232</v>
       </c>
     </row>
     <row r="90">
@@ -25990,25 +26005,25 @@
         <v>32934</v>
       </c>
       <c r="H94" t="n">
-        <v>2360</v>
+        <v>2259.3572</v>
       </c>
       <c r="I94" t="n">
-        <v>1000</v>
+        <v>970.6667</v>
       </c>
       <c r="J94" t="n">
-        <v>2632</v>
+        <v>2610.818</v>
       </c>
       <c r="K94" t="n">
-        <v>1000</v>
+        <v>970.6667</v>
       </c>
       <c r="L94" t="n">
-        <v>2632</v>
+        <v>2610.818</v>
       </c>
       <c r="M94" t="n">
-        <v>-549</v>
+        <v>-519.6667</v>
       </c>
       <c r="N94" t="n">
-        <v>-3534</v>
+        <v>-3512.818</v>
       </c>
     </row>
     <row r="95">
@@ -26235,22 +26250,22 @@
         <v>36198</v>
       </c>
       <c r="H99" t="n">
-        <v>4274.2</v>
+        <v>4414.8945</v>
       </c>
       <c r="I99" t="n">
-        <v>1375.5555</v>
+        <v>1347.375</v>
       </c>
       <c r="J99" t="n">
         <v>6645.8184</v>
       </c>
       <c r="K99" t="n">
-        <v>1375.5555</v>
+        <v>1347.375</v>
       </c>
       <c r="L99" t="n">
         <v>6645.8184</v>
       </c>
       <c r="M99" t="n">
-        <v>122.4445000000001</v>
+        <v>150.625</v>
       </c>
       <c r="N99" t="n">
         <v>-9641.8184</v>
@@ -26584,22 +26599,19 @@
         <v>18661</v>
       </c>
       <c r="H106" t="n">
-        <v>43332.668</v>
+        <v>0</v>
       </c>
       <c r="I106" t="n">
         <v>0</v>
       </c>
       <c r="J106" t="n">
-        <v>43332.668</v>
+        <v>0</v>
       </c>
       <c r="K106" t="n">
         <v>0</v>
       </c>
       <c r="L106" t="n">
-        <v>43332.668</v>
-      </c>
-      <c r="N106" t="n">
-        <v>-45856.668</v>
+        <v>0</v>
       </c>
     </row>
     <row r="107">
@@ -26918,22 +26930,22 @@
         <v>27691</v>
       </c>
       <c r="H113" t="n">
-        <v>2673.3635</v>
+        <v>2670.4546</v>
       </c>
       <c r="I113" t="n">
-        <v>1270.7142</v>
+        <v>1261.5714</v>
       </c>
       <c r="J113" t="n">
         <v>3327.9333</v>
       </c>
       <c r="K113" t="n">
-        <v>1270.7142</v>
+        <v>1261.5714</v>
       </c>
       <c r="L113" t="n">
         <v>3327.9333</v>
       </c>
       <c r="M113" t="n">
-        <v>899.2858000000001</v>
+        <v>908.4286</v>
       </c>
       <c r="N113" t="n">
         <v>-7667.933300000001</v>
@@ -27537,22 +27549,22 @@
         <v>36198</v>
       </c>
       <c r="H126" t="n">
-        <v>4274.2</v>
+        <v>4414.8945</v>
       </c>
       <c r="I126" t="n">
-        <v>1375.5555</v>
+        <v>1347.375</v>
       </c>
       <c r="J126" t="n">
         <v>6645.8184</v>
       </c>
       <c r="K126" t="n">
-        <v>4126.666499999999</v>
+        <v>4042.125</v>
       </c>
       <c r="L126" t="n">
         <v>19937.4552</v>
       </c>
       <c r="M126" t="n">
-        <v>-1656.666499999999</v>
+        <v>-1572.125</v>
       </c>
       <c r="N126" t="n">
         <v>-24877.4552</v>
@@ -27825,25 +27837,25 @@
         <v>44019</v>
       </c>
       <c r="H132" t="n">
-        <v>822.59375</v>
+        <v>1262.2</v>
       </c>
       <c r="I132" t="n">
-        <v>750.4074000000001</v>
+        <v>1119.9166</v>
       </c>
       <c r="J132" t="n">
-        <v>1212.4</v>
+        <v>1831.3334</v>
       </c>
       <c r="K132" t="n">
-        <v>2251.2222</v>
+        <v>3359.7498</v>
       </c>
       <c r="L132" t="n">
-        <v>3637.2</v>
+        <v>5494.0002</v>
       </c>
       <c r="M132" t="n">
-        <v>278.7777999999998</v>
+        <v>-829.7498000000001</v>
       </c>
       <c r="N132" t="n">
-        <v>-8697.200000000001</v>
+        <v>-10554.0002</v>
       </c>
     </row>
     <row r="133">
@@ -27926,22 +27938,22 @@
         <v>44020</v>
       </c>
       <c r="H134" t="n">
-        <v>3689.125</v>
+        <v>3496.0293</v>
       </c>
       <c r="I134" t="n">
-        <v>3509.3704</v>
+        <v>3295.3794</v>
       </c>
       <c r="J134" t="n">
         <v>4659.8</v>
       </c>
       <c r="K134" t="n">
-        <v>10528.1112</v>
+        <v>9886.138199999999</v>
       </c>
       <c r="L134" t="n">
         <v>13979.4</v>
       </c>
       <c r="M134" t="n">
-        <v>-7993.111199999999</v>
+        <v>-7351.138199999999</v>
       </c>
       <c r="N134" t="n">
         <v>-19049.4</v>
@@ -28027,25 +28039,25 @@
         <v>44021</v>
       </c>
       <c r="H136" t="n">
-        <v>6503.5625</v>
+        <v>6243.4116</v>
       </c>
       <c r="I136" t="n">
-        <v>6325.5356</v>
+        <v>6176.793</v>
       </c>
       <c r="J136" t="n">
-        <v>7749.75</v>
+        <v>6629.8</v>
       </c>
       <c r="K136" t="n">
-        <v>18976.6068</v>
+        <v>18530.379</v>
       </c>
       <c r="L136" t="n">
-        <v>23249.25</v>
+        <v>19889.4</v>
       </c>
       <c r="M136" t="n">
-        <v>-16426.6068</v>
+        <v>-15980.379</v>
       </c>
       <c r="N136" t="n">
-        <v>-28349.25</v>
+        <v>-24989.4</v>
       </c>
     </row>
     <row r="137">
@@ -28921,25 +28933,22 @@
         <v>4854</v>
       </c>
       <c r="H12" t="n">
-        <v>119.61539</v>
+        <v>228</v>
       </c>
       <c r="I12" t="n">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="J12" t="n">
-        <v>138.63637</v>
+        <v>228</v>
       </c>
       <c r="K12" t="n">
-        <v>45</v>
+        <v>0</v>
       </c>
       <c r="L12" t="n">
-        <v>415.90911</v>
-      </c>
-      <c r="M12" t="n">
-        <v>128</v>
+        <v>684</v>
       </c>
       <c r="N12" t="n">
-        <v>-761.9091100000001</v>
+        <v>-1030</v>
       </c>
     </row>
     <row r="13">
@@ -30084,25 +30093,25 @@
         <v>4718</v>
       </c>
       <c r="H35" t="n">
-        <v>533.8333</v>
+        <v>1010.6</v>
       </c>
       <c r="I35" t="n">
         <v>150</v>
       </c>
       <c r="J35" t="n">
-        <v>610.6</v>
+        <v>1225.75</v>
       </c>
       <c r="K35" t="n">
         <v>450</v>
       </c>
       <c r="L35" t="n">
-        <v>1831.8</v>
+        <v>3677.25</v>
       </c>
       <c r="M35" t="n">
         <v>-162</v>
       </c>
       <c r="N35" t="n">
-        <v>-2407.8</v>
+        <v>-4253.25</v>
       </c>
     </row>
     <row r="36">
@@ -30234,25 +30243,25 @@
         <v>4860</v>
       </c>
       <c r="H38" t="n">
-        <v>441.1111</v>
+        <v>479.9375</v>
       </c>
       <c r="I38" t="n">
-        <v>111.8</v>
+        <v>107</v>
       </c>
       <c r="J38" t="n">
-        <v>567.7692</v>
+        <v>604.25</v>
       </c>
       <c r="K38" t="n">
-        <v>335.4</v>
+        <v>321</v>
       </c>
       <c r="L38" t="n">
-        <v>1703.3076</v>
+        <v>1812.75</v>
       </c>
       <c r="M38" t="n">
-        <v>11.60000000000002</v>
+        <v>26</v>
       </c>
       <c r="N38" t="n">
-        <v>-2397.3076</v>
+        <v>-2506.75</v>
       </c>
     </row>
     <row r="39">
@@ -30338,22 +30347,22 @@
         <v>4827</v>
       </c>
       <c r="H40" t="n">
-        <v>80.708336</v>
+        <v>79.55556</v>
       </c>
       <c r="I40" t="n">
-        <v>79.882355</v>
+        <v>77.545456</v>
       </c>
       <c r="J40" t="n">
         <v>82.71429000000001</v>
       </c>
       <c r="K40" t="n">
-        <v>319.52942</v>
+        <v>310.181824</v>
       </c>
       <c r="L40" t="n">
         <v>330.85716</v>
       </c>
       <c r="M40" t="n">
-        <v>-250.52942</v>
+        <v>-241.181824</v>
       </c>
       <c r="N40" t="n">
         <v>-468.85716</v>
@@ -32410,26 +32419,23 @@
         <v>12843</v>
       </c>
       <c r="H81" t="n">
-        <v>1619.2</v>
+        <v>899.5</v>
       </c>
       <c r="I81" t="n">
         <v>899.5</v>
       </c>
       <c r="J81" t="n">
-        <v>2099</v>
+        <v>0</v>
       </c>
       <c r="K81" t="n">
         <v>2698.5</v>
       </c>
       <c r="L81" t="n">
-        <v>6297</v>
+        <v>0</v>
       </c>
       <c r="M81" t="n">
         <v>-1575.5</v>
       </c>
-      <c r="N81" t="n">
-        <v>-8543</v>
-      </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -32563,26 +32569,23 @@
         <v>12843</v>
       </c>
       <c r="H84" t="n">
-        <v>1619.2</v>
+        <v>899.5</v>
       </c>
       <c r="I84" t="n">
         <v>899.5</v>
       </c>
       <c r="J84" t="n">
-        <v>2099</v>
+        <v>0</v>
       </c>
       <c r="K84" t="n">
         <v>8095.5</v>
       </c>
       <c r="L84" t="n">
-        <v>18891</v>
+        <v>0</v>
       </c>
       <c r="M84" t="n">
         <v>-2479.5</v>
       </c>
-      <c r="N84" t="n">
-        <v>-30123</v>
-      </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -33212,25 +33215,25 @@
         <v>19846</v>
       </c>
       <c r="H97" t="n">
-        <v>650</v>
+        <v>850</v>
       </c>
       <c r="I97" t="n">
-        <v>300</v>
+        <v>450</v>
       </c>
       <c r="J97" t="n">
-        <v>1000</v>
+        <v>1250</v>
       </c>
       <c r="K97" t="n">
-        <v>900</v>
+        <v>1350</v>
       </c>
       <c r="L97" t="n">
-        <v>3000</v>
+        <v>3750</v>
       </c>
       <c r="M97" t="n">
-        <v>-404</v>
+        <v>-854</v>
       </c>
       <c r="N97" t="n">
-        <v>-3992</v>
+        <v>-4742</v>
       </c>
     </row>
     <row r="98">
@@ -33555,25 +33558,25 @@
         <v>19807</v>
       </c>
       <c r="H104" t="n">
-        <v>1850.6666</v>
+        <v>5513</v>
       </c>
       <c r="I104" t="n">
         <v>1026</v>
       </c>
       <c r="J104" t="n">
-        <v>3500</v>
+        <v>10000</v>
       </c>
       <c r="K104" t="n">
         <v>3078</v>
       </c>
       <c r="L104" t="n">
-        <v>10500</v>
+        <v>30000</v>
       </c>
       <c r="M104" t="n">
         <v>-457</v>
       </c>
       <c r="N104" t="n">
-        <v>-15742</v>
+        <v>-35242</v>
       </c>
     </row>
     <row r="105">
@@ -33959,22 +33962,22 @@
         <v>27855</v>
       </c>
       <c r="H112" t="n">
-        <v>50590</v>
+        <v>40671.8</v>
       </c>
       <c r="I112" t="n">
-        <v>1150</v>
+        <v>1099.6666</v>
       </c>
       <c r="J112" t="n">
         <v>100030</v>
       </c>
       <c r="K112" t="n">
-        <v>3450</v>
+        <v>3298.9998</v>
       </c>
       <c r="L112" t="n">
         <v>300090</v>
       </c>
       <c r="M112" t="n">
-        <v>-2342</v>
+        <v>-2190.9998</v>
       </c>
       <c r="N112" t="n">
         <v>-302306</v>
@@ -34773,22 +34776,22 @@
         <v>41814</v>
       </c>
       <c r="H128" t="n">
-        <v>264595.5</v>
+        <v>276884</v>
       </c>
       <c r="I128" t="n">
-        <v>264595.5</v>
+        <v>276884</v>
       </c>
       <c r="J128" t="n">
         <v>0</v>
       </c>
       <c r="K128" t="n">
-        <v>793786.5</v>
+        <v>830652</v>
       </c>
       <c r="L128" t="n">
         <v>0</v>
       </c>
       <c r="M128" t="n">
-        <v>-788806.5</v>
+        <v>-825672</v>
       </c>
     </row>
     <row r="129">
@@ -35232,25 +35235,25 @@
         <v>44088</v>
       </c>
       <c r="H137" t="n">
-        <v>2648.9312</v>
+        <v>2636.862</v>
       </c>
       <c r="I137" t="n">
         <v>1319</v>
       </c>
       <c r="J137" t="n">
-        <v>3587.7058</v>
+        <v>3567.1177</v>
       </c>
       <c r="K137" t="n">
         <v>3957</v>
       </c>
       <c r="L137" t="n">
-        <v>10763.1174</v>
+        <v>10701.3531</v>
       </c>
       <c r="M137" t="n">
         <v>1143</v>
       </c>
       <c r="N137" t="n">
-        <v>-20963.1174</v>
+        <v>-20901.3531</v>
       </c>
     </row>
     <row r="138">
@@ -36337,25 +36340,25 @@
         <v>2445</v>
       </c>
       <c r="H17" t="n">
-        <v>421.85715</v>
+        <v>387</v>
       </c>
       <c r="I17" t="n">
-        <v>208</v>
+        <v>220.75</v>
       </c>
       <c r="J17" t="n">
-        <v>457.5</v>
+        <v>520</v>
       </c>
       <c r="K17" t="n">
-        <v>208</v>
+        <v>220.75</v>
       </c>
       <c r="L17" t="n">
-        <v>457.5</v>
+        <v>520</v>
       </c>
       <c r="M17" t="n">
-        <v>-40</v>
+        <v>-52.75</v>
       </c>
       <c r="N17" t="n">
-        <v>-793.5</v>
+        <v>-856</v>
       </c>
     </row>
     <row r="18">
@@ -36536,22 +36539,22 @@
         <v>4430</v>
       </c>
       <c r="H21" t="n">
-        <v>2000000</v>
+        <v>348571.44</v>
       </c>
       <c r="I21" t="n">
         <v>0</v>
       </c>
       <c r="J21" t="n">
-        <v>2000000</v>
+        <v>348571.44</v>
       </c>
       <c r="K21" t="n">
         <v>0</v>
       </c>
       <c r="L21" t="n">
-        <v>2000000</v>
+        <v>348571.44</v>
       </c>
       <c r="N21" t="n">
-        <v>-2000346</v>
+        <v>-348917.44</v>
       </c>
     </row>
     <row r="22">
@@ -36983,22 +36986,22 @@
         <v>4430</v>
       </c>
       <c r="H30" t="n">
-        <v>2000000</v>
+        <v>348571.44</v>
       </c>
       <c r="I30" t="n">
         <v>0</v>
       </c>
       <c r="J30" t="n">
-        <v>2000000</v>
+        <v>348571.44</v>
       </c>
       <c r="K30" t="n">
         <v>0</v>
       </c>
       <c r="L30" t="n">
-        <v>2000000</v>
+        <v>348571.44</v>
       </c>
       <c r="N30" t="n">
-        <v>-2000210</v>
+        <v>-348781.44</v>
       </c>
     </row>
     <row r="31">
@@ -37271,25 +37274,25 @@
         <v>4222</v>
       </c>
       <c r="H36" t="n">
-        <v>8125</v>
+        <v>10166.667</v>
       </c>
       <c r="I36" t="n">
         <v>13500</v>
       </c>
       <c r="J36" t="n">
-        <v>2750</v>
+        <v>3500</v>
       </c>
       <c r="K36" t="n">
         <v>13500</v>
       </c>
       <c r="L36" t="n">
-        <v>2750</v>
+        <v>3500</v>
       </c>
       <c r="M36" t="n">
         <v>-13015</v>
       </c>
       <c r="N36" t="n">
-        <v>-3720</v>
+        <v>-4470</v>
       </c>
     </row>
     <row r="37">
@@ -37905,22 +37908,22 @@
         <v>4232</v>
       </c>
       <c r="H49" t="n">
-        <v>25000</v>
+        <v>15000</v>
       </c>
       <c r="I49" t="n">
         <v>0</v>
       </c>
       <c r="J49" t="n">
-        <v>25000</v>
+        <v>15000</v>
       </c>
       <c r="K49" t="n">
         <v>0</v>
       </c>
       <c r="L49" t="n">
-        <v>25000</v>
+        <v>15000</v>
       </c>
       <c r="N49" t="n">
-        <v>-25368</v>
+        <v>-15368</v>
       </c>
     </row>
     <row r="50">
@@ -38052,19 +38055,22 @@
         <v>4147</v>
       </c>
       <c r="H52" t="n">
-        <v>0</v>
+        <v>40000</v>
       </c>
       <c r="I52" t="n">
         <v>0</v>
       </c>
       <c r="J52" t="n">
-        <v>0</v>
+        <v>40000</v>
       </c>
       <c r="K52" t="n">
         <v>0</v>
       </c>
       <c r="L52" t="n">
-        <v>0</v>
+        <v>40000</v>
+      </c>
+      <c r="N52" t="n">
+        <v>-40518</v>
       </c>
     </row>
     <row r="53">
@@ -39382,22 +39388,22 @@
         <v>12521</v>
       </c>
       <c r="H80" t="n">
-        <v>2671.7778</v>
+        <v>2484.6</v>
       </c>
       <c r="I80" t="n">
-        <v>2429.2</v>
+        <v>2157.6667</v>
       </c>
       <c r="J80" t="n">
         <v>2975</v>
       </c>
       <c r="K80" t="n">
-        <v>2429.2</v>
+        <v>2157.6667</v>
       </c>
       <c r="L80" t="n">
         <v>2975</v>
       </c>
       <c r="M80" t="n">
-        <v>-1431.2</v>
+        <v>-1159.6667</v>
       </c>
       <c r="N80" t="n">
         <v>-4971</v>
@@ -39526,22 +39532,22 @@
         <v>12521</v>
       </c>
       <c r="H83" t="n">
-        <v>2671.7778</v>
+        <v>2484.6</v>
       </c>
       <c r="I83" t="n">
-        <v>2429.2</v>
+        <v>2157.6667</v>
       </c>
       <c r="J83" t="n">
         <v>2975</v>
       </c>
       <c r="K83" t="n">
-        <v>12146</v>
+        <v>10788.3335</v>
       </c>
       <c r="L83" t="n">
         <v>14875</v>
       </c>
       <c r="M83" t="n">
-        <v>-7154</v>
+        <v>-5796.333500000001</v>
       </c>
       <c r="N83" t="n">
         <v>-24859</v>
@@ -41404,25 +41410,25 @@
         <v>36182</v>
       </c>
       <c r="H122" t="n">
-        <v>856.75</v>
+        <v>833.5</v>
       </c>
       <c r="I122" t="n">
-        <v>809.1111</v>
+        <v>786.2</v>
       </c>
       <c r="J122" t="n">
-        <v>999.6667</v>
+        <v>951.75</v>
       </c>
       <c r="K122" t="n">
-        <v>2427.3333</v>
+        <v>2358.6</v>
       </c>
       <c r="L122" t="n">
-        <v>2999.0001</v>
+        <v>2855.25</v>
       </c>
       <c r="M122" t="n">
-        <v>22.66670000000022</v>
+        <v>91.39999999999964</v>
       </c>
       <c r="N122" t="n">
-        <v>-7899.0001</v>
+        <v>-7755.25</v>
       </c>
     </row>
     <row r="123">
@@ -41600,25 +41606,25 @@
         <v>36184</v>
       </c>
       <c r="H126" t="n">
-        <v>3577.647</v>
+        <v>4077.3572</v>
       </c>
       <c r="I126" t="n">
-        <v>1781.3636</v>
+        <v>1898.1111</v>
       </c>
       <c r="J126" t="n">
-        <v>6870.8335</v>
+        <v>8000</v>
       </c>
       <c r="K126" t="n">
-        <v>5344.0908</v>
+        <v>5694.3333</v>
       </c>
       <c r="L126" t="n">
-        <v>20612.5005</v>
+        <v>24000</v>
       </c>
       <c r="M126" t="n">
-        <v>-2874.0908</v>
+        <v>-3224.3333</v>
       </c>
       <c r="N126" t="n">
-        <v>-25552.5005</v>
+        <v>-28940</v>
       </c>
     </row>
     <row r="127">
@@ -41888,22 +41894,22 @@
         <v>44008</v>
       </c>
       <c r="H132" t="n">
-        <v>1948.5918</v>
+        <v>1856.9615</v>
       </c>
       <c r="I132" t="n">
-        <v>1771.6744</v>
+        <v>1679.6305</v>
       </c>
       <c r="J132" t="n">
         <v>3216.5</v>
       </c>
       <c r="K132" t="n">
-        <v>5315.023200000001</v>
+        <v>5038.8915</v>
       </c>
       <c r="L132" t="n">
         <v>9649.5</v>
       </c>
       <c r="M132" t="n">
-        <v>-2785.023200000001</v>
+        <v>-2508.8915</v>
       </c>
       <c r="N132" t="n">
         <v>-14709.5</v>
@@ -41940,22 +41946,22 @@
         <v>41854</v>
       </c>
       <c r="H133" t="n">
-        <v>275000</v>
+        <v>250000</v>
       </c>
       <c r="I133" t="n">
         <v>0</v>
       </c>
       <c r="J133" t="n">
-        <v>275000</v>
+        <v>250000</v>
       </c>
       <c r="K133" t="n">
         <v>0</v>
       </c>
       <c r="L133" t="n">
-        <v>275000</v>
+        <v>250000</v>
       </c>
       <c r="N133" t="n">
-        <v>-285120</v>
+        <v>-260120</v>
       </c>
     </row>
     <row r="134">
@@ -42464,22 +42470,22 @@
         <v>2631</v>
       </c>
       <c r="H2" t="n">
-        <v>19428.715</v>
+        <v>15889</v>
       </c>
       <c r="I2" t="n">
-        <v>19991</v>
+        <v>8997</v>
       </c>
       <c r="J2" t="n">
         <v>19335</v>
       </c>
       <c r="K2" t="n">
-        <v>19991</v>
+        <v>8997</v>
       </c>
       <c r="L2" t="n">
         <v>19335</v>
       </c>
       <c r="M2" t="n">
-        <v>-19879</v>
+        <v>-8885</v>
       </c>
       <c r="N2" t="n">
         <v>-19559</v>
@@ -42709,22 +42715,22 @@
         <v>36249</v>
       </c>
       <c r="H7" t="n">
-        <v>4878.8335</v>
+        <v>4763.6</v>
       </c>
       <c r="I7" t="n">
-        <v>2259.6</v>
+        <v>2216</v>
       </c>
       <c r="J7" t="n">
         <v>5568.1055</v>
       </c>
       <c r="K7" t="n">
-        <v>2259.6</v>
+        <v>2216</v>
       </c>
       <c r="L7" t="n">
         <v>5568.1055</v>
       </c>
       <c r="M7" t="n">
-        <v>-2147.6</v>
+        <v>-2104</v>
       </c>
       <c r="N7" t="n">
         <v>-5792.1055</v>
@@ -43003,22 +43009,22 @@
         <v>3546</v>
       </c>
       <c r="H13" t="n">
-        <v>29994.445</v>
+        <v>29995</v>
       </c>
       <c r="I13" t="n">
-        <v>29994.445</v>
+        <v>29995</v>
       </c>
       <c r="J13" t="n">
         <v>0</v>
       </c>
       <c r="K13" t="n">
-        <v>29994.445</v>
+        <v>29995</v>
       </c>
       <c r="L13" t="n">
         <v>0</v>
       </c>
       <c r="M13" t="n">
-        <v>-29854.445</v>
+        <v>-29855</v>
       </c>
     </row>
     <row r="14">
@@ -43285,22 +43291,22 @@
         <v>2229</v>
       </c>
       <c r="H19" t="n">
-        <v>3175</v>
+        <v>4166.6665</v>
       </c>
       <c r="I19" t="n">
-        <v>1733.3334</v>
+        <v>2500</v>
       </c>
       <c r="J19" t="n">
         <v>7500</v>
       </c>
       <c r="K19" t="n">
-        <v>1733.3334</v>
+        <v>2500</v>
       </c>
       <c r="L19" t="n">
         <v>7500</v>
       </c>
       <c r="M19" t="n">
-        <v>-1563.3334</v>
+        <v>-2330</v>
       </c>
       <c r="N19" t="n">
         <v>-7840</v>
@@ -43438,25 +43444,25 @@
         <v>5277</v>
       </c>
       <c r="H22" t="n">
-        <v>3110</v>
+        <v>3081.5</v>
       </c>
       <c r="I22" t="n">
-        <v>2926.2856</v>
+        <v>2818.111</v>
       </c>
       <c r="J22" t="n">
-        <v>3238.6</v>
+        <v>3344.889</v>
       </c>
       <c r="K22" t="n">
-        <v>2926.2856</v>
+        <v>2818.111</v>
       </c>
       <c r="L22" t="n">
-        <v>3238.6</v>
+        <v>3344.889</v>
       </c>
       <c r="M22" t="n">
-        <v>-2631.2856</v>
+        <v>-2523.111</v>
       </c>
       <c r="N22" t="n">
-        <v>-3828.6</v>
+        <v>-3934.889</v>
       </c>
     </row>
     <row r="23">
@@ -43588,22 +43594,22 @@
         <v>3547</v>
       </c>
       <c r="H25" t="n">
-        <v>9251</v>
+        <v>9999</v>
       </c>
       <c r="I25" t="n">
-        <v>8503</v>
+        <v>9999</v>
       </c>
       <c r="J25" t="n">
         <v>9999</v>
       </c>
       <c r="K25" t="n">
-        <v>8503</v>
+        <v>9999</v>
       </c>
       <c r="L25" t="n">
         <v>9999</v>
       </c>
       <c r="M25" t="n">
-        <v>-8273</v>
+        <v>-9769</v>
       </c>
       <c r="N25" t="n">
         <v>-10459</v>
@@ -43689,25 +43695,25 @@
         <v>5277</v>
       </c>
       <c r="H27" t="n">
-        <v>3110</v>
+        <v>3081.5</v>
       </c>
       <c r="I27" t="n">
-        <v>2926.2856</v>
+        <v>2818.111</v>
       </c>
       <c r="J27" t="n">
-        <v>3238.6</v>
+        <v>3344.889</v>
       </c>
       <c r="K27" t="n">
-        <v>2926.2856</v>
+        <v>2818.111</v>
       </c>
       <c r="L27" t="n">
-        <v>3238.6</v>
+        <v>3344.889</v>
       </c>
       <c r="M27" t="n">
-        <v>-2819.2856</v>
+        <v>-2711.111</v>
       </c>
       <c r="N27" t="n">
-        <v>-3452.6</v>
+        <v>-3558.889</v>
       </c>
     </row>
     <row r="28">
@@ -43986,22 +43992,19 @@
         <v>4106</v>
       </c>
       <c r="H33" t="n">
-        <v>20000</v>
+        <v>0</v>
       </c>
       <c r="I33" t="n">
-        <v>20000</v>
+        <v>0</v>
       </c>
       <c r="J33" t="n">
         <v>0</v>
       </c>
       <c r="K33" t="n">
-        <v>20000</v>
+        <v>0</v>
       </c>
       <c r="L33" t="n">
         <v>0</v>
-      </c>
-      <c r="M33" t="n">
-        <v>-19710</v>
       </c>
     </row>
     <row r="34">
@@ -44136,19 +44139,22 @@
         <v>34261</v>
       </c>
       <c r="H36" t="n">
-        <v>0</v>
+        <v>88000</v>
       </c>
       <c r="I36" t="n">
-        <v>0</v>
+        <v>88000</v>
       </c>
       <c r="J36" t="n">
         <v>0</v>
       </c>
       <c r="K36" t="n">
-        <v>0</v>
+        <v>88000</v>
       </c>
       <c r="L36" t="n">
         <v>0</v>
+      </c>
+      <c r="M36" t="n">
+        <v>-87438</v>
       </c>
     </row>
     <row r="37">
@@ -44320,25 +44326,25 @@
         <v>36248</v>
       </c>
       <c r="H40" t="n">
-        <v>2320.0908</v>
+        <v>2326.75</v>
       </c>
       <c r="I40" t="n">
         <v>1669</v>
       </c>
       <c r="J40" t="n">
-        <v>5250</v>
+        <v>4300</v>
       </c>
       <c r="K40" t="n">
         <v>1669</v>
       </c>
       <c r="L40" t="n">
-        <v>5250</v>
+        <v>4300</v>
       </c>
       <c r="M40" t="n">
         <v>-1533</v>
       </c>
       <c r="N40" t="n">
-        <v>-5522</v>
+        <v>-4572</v>
       </c>
     </row>
     <row r="41">
@@ -44562,22 +44568,22 @@
         <v>3851</v>
       </c>
       <c r="H45" t="n">
-        <v>14851.08</v>
+        <v>14094.958</v>
       </c>
       <c r="I45" t="n">
-        <v>13803.208</v>
+        <v>12968.652</v>
       </c>
       <c r="J45" t="n">
         <v>40000</v>
       </c>
       <c r="K45" t="n">
-        <v>13803.208</v>
+        <v>12968.652</v>
       </c>
       <c r="L45" t="n">
         <v>40000</v>
       </c>
       <c r="M45" t="n">
-        <v>-13396.208</v>
+        <v>-12561.652</v>
       </c>
       <c r="N45" t="n">
         <v>-40814</v>
@@ -44614,25 +44620,25 @@
         <v>5282</v>
       </c>
       <c r="H46" t="n">
-        <v>3073.1428</v>
+        <v>3464</v>
       </c>
       <c r="I46" t="n">
-        <v>1022</v>
+        <v>999.75</v>
       </c>
       <c r="J46" t="n">
-        <v>4335.385</v>
+        <v>4168.0713</v>
       </c>
       <c r="K46" t="n">
-        <v>1022</v>
+        <v>999.75</v>
       </c>
       <c r="L46" t="n">
-        <v>4335.385</v>
+        <v>4168.0713</v>
       </c>
       <c r="M46" t="n">
-        <v>-834</v>
+        <v>-811.75</v>
       </c>
       <c r="N46" t="n">
-        <v>-4711.385</v>
+        <v>-4544.0713</v>
       </c>
     </row>
     <row r="47">
@@ -44712,22 +44718,22 @@
         <v>3625</v>
       </c>
       <c r="H48" t="n">
-        <v>2611.6667</v>
+        <v>2387.6</v>
       </c>
       <c r="I48" t="n">
-        <v>2611.6667</v>
+        <v>2387.6</v>
       </c>
       <c r="J48" t="n">
         <v>0</v>
       </c>
       <c r="K48" t="n">
-        <v>2611.6667</v>
+        <v>2387.6</v>
       </c>
       <c r="L48" t="n">
         <v>0</v>
       </c>
       <c r="M48" t="n">
-        <v>-1950.6667</v>
+        <v>-1726.6</v>
       </c>
     </row>
     <row r="49">
@@ -44859,22 +44865,19 @@
         <v>3423</v>
       </c>
       <c r="H51" t="n">
-        <v>20000</v>
+        <v>0</v>
       </c>
       <c r="I51" t="n">
         <v>0</v>
       </c>
       <c r="J51" t="n">
-        <v>20000</v>
+        <v>0</v>
       </c>
       <c r="K51" t="n">
         <v>0</v>
       </c>
       <c r="L51" t="n">
-        <v>20000</v>
-      </c>
-      <c r="N51" t="n">
-        <v>-20956</v>
+        <v>0</v>
       </c>
     </row>
     <row r="52">
@@ -45346,22 +45349,22 @@
         <v>27740</v>
       </c>
       <c r="H61" t="n">
-        <v>47627084</v>
+        <v>45462270</v>
       </c>
       <c r="I61" t="n">
-        <v>58832040</v>
+        <v>55563660</v>
       </c>
       <c r="J61" t="n">
         <v>6020.75</v>
       </c>
       <c r="K61" t="n">
-        <v>58832040</v>
+        <v>55563660</v>
       </c>
       <c r="L61" t="n">
         <v>6020.75</v>
       </c>
       <c r="M61" t="n">
-        <v>-58831838</v>
+        <v>-55563458</v>
       </c>
       <c r="N61" t="n">
         <v>-6424.75</v>
@@ -45698,22 +45701,22 @@
         <v>12563</v>
       </c>
       <c r="H68" t="n">
-        <v>2100.5</v>
+        <v>2624.75</v>
       </c>
       <c r="I68" t="n">
-        <v>1900</v>
+        <v>2748</v>
       </c>
       <c r="J68" t="n">
         <v>2501.5</v>
       </c>
       <c r="K68" t="n">
-        <v>1900</v>
+        <v>2748</v>
       </c>
       <c r="L68" t="n">
         <v>2501.5</v>
       </c>
       <c r="M68" t="n">
-        <v>-1151</v>
+        <v>-1999</v>
       </c>
       <c r="N68" t="n">
         <v>-3999.5</v>
@@ -45848,22 +45851,22 @@
         <v>12563</v>
       </c>
       <c r="H71" t="n">
-        <v>2100.5</v>
+        <v>2624.75</v>
       </c>
       <c r="I71" t="n">
-        <v>1900</v>
+        <v>2748</v>
       </c>
       <c r="J71" t="n">
         <v>2501.5</v>
       </c>
       <c r="K71" t="n">
-        <v>9500</v>
+        <v>13740</v>
       </c>
       <c r="L71" t="n">
         <v>12507.5</v>
       </c>
       <c r="M71" t="n">
-        <v>-5756</v>
+        <v>-9996</v>
       </c>
       <c r="N71" t="n">
         <v>-19995.5</v>
@@ -46384,25 +46387,25 @@
         <v>12565</v>
       </c>
       <c r="H82" t="n">
-        <v>1407.1666</v>
+        <v>1434.0588</v>
       </c>
       <c r="I82" t="n">
         <v>997.6667</v>
       </c>
       <c r="J82" t="n">
-        <v>1816.6666</v>
+        <v>1925</v>
       </c>
       <c r="K82" t="n">
         <v>997.6667</v>
       </c>
       <c r="L82" t="n">
-        <v>1816.6666</v>
+        <v>1925</v>
       </c>
       <c r="M82" t="n">
         <v>-636.6667</v>
       </c>
       <c r="N82" t="n">
-        <v>-2538.6666</v>
+        <v>-2647</v>
       </c>
     </row>
     <row r="83">
@@ -46534,25 +46537,25 @@
         <v>12565</v>
       </c>
       <c r="H85" t="n">
-        <v>1407.1666</v>
+        <v>1434.0588</v>
       </c>
       <c r="I85" t="n">
         <v>997.6667</v>
       </c>
       <c r="J85" t="n">
-        <v>1816.6666</v>
+        <v>1925</v>
       </c>
       <c r="K85" t="n">
         <v>997.6667</v>
       </c>
       <c r="L85" t="n">
-        <v>1816.6666</v>
+        <v>1925</v>
       </c>
       <c r="M85" t="n">
         <v>250.3333</v>
       </c>
       <c r="N85" t="n">
-        <v>-4312.6666</v>
+        <v>-4421</v>
       </c>
     </row>
     <row r="86">
@@ -47266,25 +47269,25 @@
         <v>19995</v>
       </c>
       <c r="H100" t="n">
-        <v>1723.75</v>
+        <v>1749</v>
       </c>
       <c r="I100" t="n">
-        <v>1449.75</v>
+        <v>1499.5</v>
       </c>
       <c r="J100" t="n">
-        <v>1997.75</v>
+        <v>1998.5</v>
       </c>
       <c r="K100" t="n">
-        <v>1449.75</v>
+        <v>1499.5</v>
       </c>
       <c r="L100" t="n">
-        <v>1997.75</v>
+        <v>1998.5</v>
       </c>
       <c r="M100" t="n">
-        <v>-908.75</v>
+        <v>-958.5</v>
       </c>
       <c r="N100" t="n">
-        <v>-3079.75</v>
+        <v>-3080.5</v>
       </c>
     </row>
     <row r="101">
@@ -47554,22 +47557,22 @@
         <v>18713</v>
       </c>
       <c r="H106" t="n">
-        <v>3353330.8</v>
+        <v>3359333</v>
       </c>
       <c r="I106" t="n">
         <v>0</v>
       </c>
       <c r="J106" t="n">
-        <v>3353330.8</v>
+        <v>3359333</v>
       </c>
       <c r="K106" t="n">
         <v>0</v>
       </c>
       <c r="L106" t="n">
-        <v>3353330.8</v>
+        <v>3359333</v>
       </c>
       <c r="N106" t="n">
-        <v>-3355854.8</v>
+        <v>-3361857</v>
       </c>
     </row>
     <row r="107">
@@ -47652,25 +47655,19 @@
         <v>25655</v>
       </c>
       <c r="H108" t="n">
-        <v>39997</v>
+        <v>0</v>
       </c>
       <c r="I108" t="n">
-        <v>39999</v>
+        <v>0</v>
       </c>
       <c r="J108" t="n">
-        <v>39995</v>
+        <v>0</v>
       </c>
       <c r="K108" t="n">
-        <v>39999</v>
+        <v>0</v>
       </c>
       <c r="L108" t="n">
-        <v>39995</v>
-      </c>
-      <c r="M108" t="n">
-        <v>-36159</v>
-      </c>
-      <c r="N108" t="n">
-        <v>-47675</v>
+        <v>0</v>
       </c>
     </row>
     <row r="109">
@@ -47894,22 +47891,22 @@
         <v>27740</v>
       </c>
       <c r="H113" t="n">
-        <v>47627084</v>
+        <v>45462270</v>
       </c>
       <c r="I113" t="n">
-        <v>58832040</v>
+        <v>55563660</v>
       </c>
       <c r="J113" t="n">
         <v>6020.75</v>
       </c>
       <c r="K113" t="n">
-        <v>58832040</v>
+        <v>55563660</v>
       </c>
       <c r="L113" t="n">
         <v>6020.75</v>
       </c>
       <c r="M113" t="n">
-        <v>-58829870</v>
+        <v>-55561490</v>
       </c>
       <c r="N113" t="n">
         <v>-10360.75</v>
@@ -48516,22 +48513,22 @@
         <v>36249</v>
       </c>
       <c r="H126" t="n">
-        <v>4878.8335</v>
+        <v>4763.6</v>
       </c>
       <c r="I126" t="n">
-        <v>2259.6</v>
+        <v>2216</v>
       </c>
       <c r="J126" t="n">
         <v>5568.1055</v>
       </c>
       <c r="K126" t="n">
-        <v>6778.799999999999</v>
+        <v>6648</v>
       </c>
       <c r="L126" t="n">
         <v>16704.3165</v>
       </c>
       <c r="M126" t="n">
-        <v>-4308.799999999999</v>
+        <v>-4178</v>
       </c>
       <c r="N126" t="n">
         <v>-21644.3165</v>
@@ -48663,22 +48660,19 @@
         <v>35433</v>
       </c>
       <c r="H129" t="n">
-        <v>60000</v>
+        <v>0</v>
       </c>
       <c r="I129" t="n">
         <v>0</v>
       </c>
       <c r="J129" t="n">
-        <v>60000</v>
+        <v>0</v>
       </c>
       <c r="K129" t="n">
         <v>0</v>
       </c>
       <c r="L129" t="n">
-        <v>60000</v>
-      </c>
-      <c r="N129" t="n">
-        <v>-70000</v>
+        <v>0</v>
       </c>
     </row>
     <row r="130">
@@ -48807,22 +48801,22 @@
         <v>44058</v>
       </c>
       <c r="H132" t="n">
-        <v>2484.5</v>
+        <v>2439.7742</v>
       </c>
       <c r="I132" t="n">
-        <v>1706.65</v>
+        <v>1677.6666</v>
       </c>
       <c r="J132" t="n">
         <v>4040.2</v>
       </c>
       <c r="K132" t="n">
-        <v>5119.950000000001</v>
+        <v>5032.9998</v>
       </c>
       <c r="L132" t="n">
         <v>12120.6</v>
       </c>
       <c r="M132" t="n">
-        <v>-2589.950000000001</v>
+        <v>-2502.9998</v>
       </c>
       <c r="N132" t="n">
         <v>-17180.6</v>
@@ -49003,22 +48997,22 @@
         <v>44060</v>
       </c>
       <c r="H136" t="n">
-        <v>3602.4324</v>
+        <v>3734.9143</v>
       </c>
       <c r="I136" t="n">
-        <v>2216.7</v>
+        <v>2297.8044</v>
       </c>
       <c r="J136" t="n">
         <v>6489.375</v>
       </c>
       <c r="K136" t="n">
-        <v>6650.099999999999</v>
+        <v>6893.4132</v>
       </c>
       <c r="L136" t="n">
         <v>19468.125</v>
       </c>
       <c r="M136" t="n">
-        <v>-4100.099999999999</v>
+        <v>-4343.4132</v>
       </c>
       <c r="N136" t="n">
         <v>-24568.125</v>
@@ -49928,22 +49922,22 @@
         <v>3008</v>
       </c>
       <c r="H13" t="n">
-        <v>255</v>
+        <v>4999</v>
       </c>
       <c r="I13" t="n">
-        <v>255</v>
+        <v>0</v>
       </c>
       <c r="J13" t="n">
-        <v>0</v>
+        <v>4999</v>
       </c>
       <c r="K13" t="n">
-        <v>255</v>
+        <v>0</v>
       </c>
       <c r="L13" t="n">
-        <v>0</v>
-      </c>
-      <c r="M13" t="n">
-        <v>-115</v>
+        <v>4999</v>
+      </c>
+      <c r="N13" t="n">
+        <v>-5279</v>
       </c>
     </row>
     <row r="14">
@@ -50026,22 +50020,22 @@
         <v>2670</v>
       </c>
       <c r="H15" t="n">
-        <v>15403.8</v>
+        <v>20004.334</v>
       </c>
       <c r="I15" t="n">
-        <v>12335</v>
+        <v>19999</v>
       </c>
       <c r="J15" t="n">
         <v>20007</v>
       </c>
       <c r="K15" t="n">
-        <v>12335</v>
+        <v>19999</v>
       </c>
       <c r="L15" t="n">
         <v>20007</v>
       </c>
       <c r="M15" t="n">
-        <v>-12047</v>
+        <v>-19711</v>
       </c>
       <c r="N15" t="n">
         <v>-20583</v>
@@ -50902,22 +50896,25 @@
         <v>2734</v>
       </c>
       <c r="H33" t="n">
-        <v>15011</v>
+        <v>4503.1665</v>
       </c>
       <c r="I33" t="n">
-        <v>15011</v>
+        <v>11509.5</v>
       </c>
       <c r="J33" t="n">
-        <v>0</v>
+        <v>1000</v>
       </c>
       <c r="K33" t="n">
-        <v>15011</v>
+        <v>11509.5</v>
       </c>
       <c r="L33" t="n">
-        <v>0</v>
+        <v>1000</v>
       </c>
       <c r="M33" t="n">
-        <v>-14761</v>
+        <v>-11259.5</v>
+      </c>
+      <c r="N33" t="n">
+        <v>-1500</v>
       </c>
     </row>
     <row r="34">
@@ -51046,22 +51043,25 @@
         <v>2734</v>
       </c>
       <c r="H36" t="n">
-        <v>15011</v>
+        <v>4503.1665</v>
       </c>
       <c r="I36" t="n">
-        <v>15011</v>
+        <v>11509.5</v>
       </c>
       <c r="J36" t="n">
-        <v>0</v>
+        <v>1000</v>
       </c>
       <c r="K36" t="n">
-        <v>15011</v>
+        <v>11509.5</v>
       </c>
       <c r="L36" t="n">
-        <v>0</v>
+        <v>1000</v>
       </c>
       <c r="M36" t="n">
-        <v>-14761</v>
+        <v>-11259.5</v>
+      </c>
+      <c r="N36" t="n">
+        <v>-1500</v>
       </c>
     </row>
     <row r="37">
@@ -51095,22 +51095,22 @@
         <v>3351</v>
       </c>
       <c r="H37" t="n">
-        <v>20342</v>
+        <v>21013</v>
       </c>
       <c r="I37" t="n">
-        <v>20342</v>
+        <v>21013</v>
       </c>
       <c r="J37" t="n">
         <v>0</v>
       </c>
       <c r="K37" t="n">
-        <v>20342</v>
+        <v>21013</v>
       </c>
       <c r="L37" t="n">
         <v>0</v>
       </c>
       <c r="M37" t="n">
-        <v>-20139</v>
+        <v>-20810</v>
       </c>
     </row>
     <row r="38">
@@ -51190,25 +51190,25 @@
         <v>3106</v>
       </c>
       <c r="H39" t="n">
-        <v>32532</v>
+        <v>33772.25</v>
       </c>
       <c r="I39" t="n">
-        <v>30042.334</v>
+        <v>30044</v>
       </c>
       <c r="J39" t="n">
-        <v>40001</v>
+        <v>37500.5</v>
       </c>
       <c r="K39" t="n">
-        <v>30042.334</v>
+        <v>30044</v>
       </c>
       <c r="L39" t="n">
-        <v>40001</v>
+        <v>37500.5</v>
       </c>
       <c r="M39" t="n">
-        <v>-29629.334</v>
+        <v>-29631</v>
       </c>
       <c r="N39" t="n">
-        <v>-40827</v>
+        <v>-38326.5</v>
       </c>
     </row>
     <row r="40">
@@ -51242,25 +51242,25 @@
         <v>3601</v>
       </c>
       <c r="H40" t="n">
-        <v>18348.666</v>
+        <v>21658.666</v>
       </c>
       <c r="I40" t="n">
-        <v>15022.5</v>
+        <v>15025</v>
       </c>
       <c r="J40" t="n">
-        <v>25001</v>
+        <v>24975.5</v>
       </c>
       <c r="K40" t="n">
-        <v>15022.5</v>
+        <v>15025</v>
       </c>
       <c r="L40" t="n">
-        <v>25001</v>
+        <v>24975.5</v>
       </c>
       <c r="M40" t="n">
-        <v>-14873.5</v>
+        <v>-14876</v>
       </c>
       <c r="N40" t="n">
-        <v>-25299</v>
+        <v>-25273.5</v>
       </c>
     </row>
     <row r="41">
@@ -51343,22 +51343,22 @@
         <v>3372</v>
       </c>
       <c r="H42" t="n">
-        <v>23520.75</v>
+        <v>26022</v>
       </c>
       <c r="I42" t="n">
-        <v>21361</v>
+        <v>22044</v>
       </c>
       <c r="J42" t="n">
         <v>30000</v>
       </c>
       <c r="K42" t="n">
-        <v>21361</v>
+        <v>22044</v>
       </c>
       <c r="L42" t="n">
         <v>30000</v>
       </c>
       <c r="M42" t="n">
-        <v>-20983</v>
+        <v>-21666</v>
       </c>
       <c r="N42" t="n">
         <v>-30756</v>
@@ -51686,22 +51686,25 @@
         <v>3397</v>
       </c>
       <c r="H49" t="n">
-        <v>25070</v>
+        <v>23345</v>
       </c>
       <c r="I49" t="n">
-        <v>25070</v>
+        <v>23214</v>
       </c>
       <c r="J49" t="n">
-        <v>0</v>
+        <v>24000</v>
       </c>
       <c r="K49" t="n">
-        <v>25070</v>
+        <v>23214</v>
       </c>
       <c r="L49" t="n">
-        <v>0</v>
+        <v>24000</v>
       </c>
       <c r="M49" t="n">
-        <v>-24840</v>
+        <v>-22984</v>
+      </c>
+      <c r="N49" t="n">
+        <v>-24460</v>
       </c>
     </row>
     <row r="50">
@@ -51940,22 +51943,22 @@
         <v>3413</v>
       </c>
       <c r="H54" t="n">
-        <v>46781.715</v>
+        <v>44694.266</v>
       </c>
       <c r="I54" t="n">
-        <v>18070</v>
+        <v>16770</v>
       </c>
       <c r="J54" t="n">
         <v>48990.31</v>
       </c>
       <c r="K54" t="n">
-        <v>18070</v>
+        <v>16770</v>
       </c>
       <c r="L54" t="n">
         <v>48990.31</v>
       </c>
       <c r="M54" t="n">
-        <v>-17550</v>
+        <v>-16250</v>
       </c>
       <c r="N54" t="n">
         <v>-50030.31</v>
@@ -52326,25 +52329,25 @@
         <v>12589</v>
       </c>
       <c r="H62" t="n">
-        <v>5287.28</v>
+        <v>5000.893</v>
       </c>
       <c r="I62" t="n">
-        <v>3375.2</v>
+        <v>3102.7144</v>
       </c>
       <c r="J62" t="n">
-        <v>5765.3</v>
+        <v>5633.619</v>
       </c>
       <c r="K62" t="n">
-        <v>3375.2</v>
+        <v>3102.7144</v>
       </c>
       <c r="L62" t="n">
-        <v>5765.3</v>
+        <v>5633.619</v>
       </c>
       <c r="M62" t="n">
-        <v>-2751.2</v>
+        <v>-2478.7144</v>
       </c>
       <c r="N62" t="n">
-        <v>-7013.3</v>
+        <v>-6881.619</v>
       </c>
     </row>
     <row r="63">
@@ -52473,25 +52476,25 @@
         <v>12589</v>
       </c>
       <c r="H65" t="n">
-        <v>5287.28</v>
+        <v>5000.893</v>
       </c>
       <c r="I65" t="n">
-        <v>3375.2</v>
+        <v>3102.7144</v>
       </c>
       <c r="J65" t="n">
-        <v>5765.3</v>
+        <v>5633.619</v>
       </c>
       <c r="K65" t="n">
-        <v>16876</v>
+        <v>15513.572</v>
       </c>
       <c r="L65" t="n">
-        <v>28826.5</v>
+        <v>28168.095</v>
       </c>
       <c r="M65" t="n">
-        <v>-13756</v>
+        <v>-12393.572</v>
       </c>
       <c r="N65" t="n">
-        <v>-35066.5</v>
+        <v>-34408.095</v>
       </c>
     </row>
     <row r="66">
@@ -52963,22 +52966,22 @@
         <v>11957</v>
       </c>
       <c r="H75" t="n">
-        <v>55000</v>
+        <v>54999.5</v>
       </c>
       <c r="I75" t="n">
-        <v>55000</v>
+        <v>54999.5</v>
       </c>
       <c r="J75" t="n">
         <v>0</v>
       </c>
       <c r="K75" t="n">
-        <v>55000</v>
+        <v>54999.5</v>
       </c>
       <c r="L75" t="n">
         <v>0</v>
       </c>
       <c r="M75" t="n">
-        <v>-54064</v>
+        <v>-54063.5</v>
       </c>
     </row>
     <row r="76">
@@ -53107,22 +53110,22 @@
         <v>11957</v>
       </c>
       <c r="H78" t="n">
-        <v>55000</v>
+        <v>54999.5</v>
       </c>
       <c r="I78" t="n">
-        <v>55000</v>
+        <v>54999.5</v>
       </c>
       <c r="J78" t="n">
         <v>0</v>
       </c>
       <c r="K78" t="n">
-        <v>165000</v>
+        <v>164998.5</v>
       </c>
       <c r="L78" t="n">
         <v>0</v>
       </c>
       <c r="M78" t="n">
-        <v>-160320</v>
+        <v>-160318.5</v>
       </c>
     </row>
     <row r="79">
@@ -53248,25 +53251,25 @@
         <v>12596</v>
       </c>
       <c r="H81" t="n">
-        <v>7264.1577</v>
+        <v>7884.7646</v>
       </c>
       <c r="I81" t="n">
-        <v>5321.3335</v>
+        <v>5990</v>
       </c>
       <c r="J81" t="n">
-        <v>8160.846</v>
+        <v>8674.25</v>
       </c>
       <c r="K81" t="n">
-        <v>10642.667</v>
+        <v>11980</v>
       </c>
       <c r="L81" t="n">
-        <v>16321.692</v>
+        <v>17348.5</v>
       </c>
       <c r="M81" t="n">
-        <v>-9581.666999999999</v>
+        <v>-10919</v>
       </c>
       <c r="N81" t="n">
-        <v>-18443.692</v>
+        <v>-19470.5</v>
       </c>
     </row>
     <row r="82">
@@ -53392,25 +53395,25 @@
         <v>12596</v>
       </c>
       <c r="H84" t="n">
-        <v>7264.1577</v>
+        <v>7884.7646</v>
       </c>
       <c r="I84" t="n">
-        <v>5321.3335</v>
+        <v>5990</v>
       </c>
       <c r="J84" t="n">
-        <v>8160.846</v>
+        <v>8674.25</v>
       </c>
       <c r="K84" t="n">
-        <v>53213.335</v>
+        <v>59900</v>
       </c>
       <c r="L84" t="n">
-        <v>81608.45999999999</v>
+        <v>86742.5</v>
       </c>
       <c r="M84" t="n">
-        <v>-47909.335</v>
+        <v>-54596</v>
       </c>
       <c r="N84" t="n">
-        <v>-92216.45999999999</v>
+        <v>-97350.5</v>
       </c>
     </row>
     <row r="85">
@@ -53980,22 +53983,22 @@
         <v>19977</v>
       </c>
       <c r="H96" t="n">
-        <v>2210.1765</v>
+        <v>1931.15</v>
       </c>
       <c r="I96" t="n">
-        <v>2269.923</v>
+        <v>1909.9375</v>
       </c>
       <c r="J96" t="n">
         <v>2016</v>
       </c>
       <c r="K96" t="n">
-        <v>2269.923</v>
+        <v>1909.9375</v>
       </c>
       <c r="L96" t="n">
         <v>2016</v>
       </c>
       <c r="M96" t="n">
-        <v>-896.9229999999998</v>
+        <v>-536.9375</v>
       </c>
       <c r="N96" t="n">
         <v>-4762</v>
@@ -54813,25 +54816,25 @@
         <v>27752</v>
       </c>
       <c r="H113" t="n">
-        <v>954.3421</v>
+        <v>925.35895</v>
       </c>
       <c r="I113" t="n">
-        <v>1127.037</v>
+        <v>1056.1724</v>
       </c>
       <c r="J113" t="n">
-        <v>530.4545000000001</v>
+        <v>546</v>
       </c>
       <c r="K113" t="n">
-        <v>3381.111</v>
+        <v>3168.5172</v>
       </c>
       <c r="L113" t="n">
-        <v>1591.3635</v>
+        <v>1638</v>
       </c>
       <c r="M113" t="n">
-        <v>-1211.111</v>
+        <v>-998.5171999999998</v>
       </c>
       <c r="N113" t="n">
-        <v>-5931.3635</v>
+        <v>-5978</v>
       </c>
     </row>
     <row r="114">
@@ -55726,22 +55729,22 @@
         <v>44029</v>
       </c>
       <c r="H132" t="n">
-        <v>3990.0356</v>
+        <v>3988.3215</v>
       </c>
       <c r="I132" t="n">
-        <v>3072.875</v>
+        <v>3069.875</v>
       </c>
       <c r="J132" t="n">
         <v>5212.9165</v>
       </c>
       <c r="K132" t="n">
-        <v>9218.625</v>
+        <v>9209.625</v>
       </c>
       <c r="L132" t="n">
         <v>15638.7495</v>
       </c>
       <c r="M132" t="n">
-        <v>-6688.625</v>
+        <v>-6679.625</v>
       </c>
       <c r="N132" t="n">
         <v>-20698.7495</v>

</xml_diff>